<commit_message>
Updated the instrument rate documents for 09/01/2026
* Sample submission form moves the UW hourly rate from 17.00 to 18.50 and the
  UW FFS rate from 34.00 to 37.00, with TSQ-Altis now at the same rate as the
  other instruments
* UWPR_Current_Rates.pdf replaces UWPR_Current_Rates.xlsx, and the "Current
  instrument rates" link in front.jsp points at the new file

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WebRoot/costcenter_resources/UWPR sample submission form.xlsx
+++ b/WebRoot/costcenter_resources/UWPR sample submission form.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PriskaStuff\UWPR costcenter\SampleSubmissionForm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Hoopmann\Documents\UWPR\Website\docs\master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4CB54E-C9F7-410F-92EB-6C625ECD2E73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CB5436B-C5AE-4556-A8EB-D3C073C96989}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2120" yWindow="4650" windowWidth="26500" windowHeight="15800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sample Submission" sheetId="3" r:id="rId1"/>
@@ -1617,9 +1617,6 @@
     <t>Exploris2</t>
   </si>
   <si>
-    <t>Rates effective 9/1/2024 subject to change without notice</t>
-  </si>
-  <si>
     <t>Enter the number of samples:</t>
   </si>
   <si>
@@ -1635,10 +1632,13 @@
     <t>Fill in as much information belwo as you know or any special instructions for the analysis:</t>
   </si>
   <si>
-    <t>Revised 9/1/25</t>
-  </si>
-  <si>
     <t>Then complete this form and upload it to your project online and email hoopmann@uw.edu to coordinate a time to drop off your samples.</t>
+  </si>
+  <si>
+    <t>Revised 9/8/2026</t>
+  </si>
+  <si>
+    <t>Rates effective 9/1/2026 subject to change without notice</t>
   </si>
 </sst>
 </file>
@@ -3423,6 +3423,69 @@
     <xf numFmtId="0" fontId="76" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="10" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="1" fontId="8" fillId="2" borderId="4" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3437,69 +3500,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="30" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="27" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="28" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="10" borderId="30" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -3823,10 +3823,10 @@
           </xdr:nvGrpSpPr>
           <xdr:grpSpPr>
             <a:xfrm>
-              <a:off x="3924300" y="10115550"/>
+              <a:off x="4108450" y="10001250"/>
               <a:ext cx="1371600" cy="209550"/>
-              <a:chOff x="2266949" y="4686300"/>
-              <a:chExt cx="1685926" cy="209550"/>
+              <a:chOff x="2266950" y="4686300"/>
+              <a:chExt cx="1685925" cy="209550"/>
             </a:xfrm>
           </xdr:grpSpPr>
           <xdr:sp macro="" textlink="">
@@ -3845,7 +3845,7 @@
             </xdr:nvSpPr>
             <xdr:spPr bwMode="auto">
               <a:xfrm>
-                <a:off x="2266949" y="4686300"/>
+                <a:off x="2266950" y="4686300"/>
                 <a:ext cx="781050" cy="209550"/>
               </a:xfrm>
               <a:prstGeom prst="rect">
@@ -3871,7 +3871,7 @@
               </a:extLst>
             </xdr:spPr>
             <xdr:txBody>
-              <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+              <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr algn="l" rtl="0">
@@ -3933,7 +3933,7 @@
               </a:extLst>
             </xdr:spPr>
             <xdr:txBody>
-              <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+              <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr algn="l" rtl="0">
@@ -3966,13 +3966,13 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>0</xdr:colOff>
           <xdr:row>34</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
+          <xdr:rowOff>69850</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>638175</xdr:colOff>
+          <xdr:colOff>641350</xdr:colOff>
           <xdr:row>34</xdr:row>
-          <xdr:rowOff>276225</xdr:rowOff>
+          <xdr:rowOff>279400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4016,7 +4016,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4046,15 +4046,15 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>733425</xdr:colOff>
+          <xdr:colOff>736600</xdr:colOff>
           <xdr:row>34</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
+          <xdr:rowOff>69850</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
           <xdr:colOff>1371600</xdr:colOff>
           <xdr:row>34</xdr:row>
-          <xdr:rowOff>276225</xdr:rowOff>
+          <xdr:rowOff>279400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4098,7 +4098,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4128,7 +4128,7 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>7</xdr:col>
-          <xdr:colOff>123825</xdr:colOff>
+          <xdr:colOff>127000</xdr:colOff>
           <xdr:row>79</xdr:row>
           <xdr:rowOff>38100</xdr:rowOff>
         </xdr:from>
@@ -4136,7 +4136,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>990600</xdr:colOff>
           <xdr:row>79</xdr:row>
-          <xdr:rowOff>257175</xdr:rowOff>
+          <xdr:rowOff>260350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4180,7 +4180,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4218,7 +4218,7 @@
           <xdr:col>8</xdr:col>
           <xdr:colOff>552450</xdr:colOff>
           <xdr:row>79</xdr:row>
-          <xdr:rowOff>257175</xdr:rowOff>
+          <xdr:rowOff>260350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4262,7 +4262,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4292,9 +4292,9 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>7</xdr:col>
-          <xdr:colOff>123825</xdr:colOff>
+          <xdr:colOff>127000</xdr:colOff>
           <xdr:row>80</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
+          <xdr:rowOff>69850</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>7</xdr:col>
@@ -4344,7 +4344,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4376,7 +4376,7 @@
           <xdr:col>7</xdr:col>
           <xdr:colOff>1066800</xdr:colOff>
           <xdr:row>80</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
+          <xdr:rowOff>69850</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>8</xdr:col>
@@ -4426,7 +4426,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4456,13 +4456,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>4</xdr:col>
-          <xdr:colOff>123825</xdr:colOff>
+          <xdr:colOff>127000</xdr:colOff>
           <xdr:row>80</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
+          <xdr:rowOff>69850</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>200025</xdr:colOff>
+          <xdr:colOff>203200</xdr:colOff>
           <xdr:row>81</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -4508,7 +4508,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4538,13 +4538,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>390525</xdr:colOff>
+          <xdr:colOff>393700</xdr:colOff>
           <xdr:row>80</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
+          <xdr:rowOff>69850</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>847725</xdr:colOff>
+          <xdr:colOff>850900</xdr:colOff>
           <xdr:row>81</xdr:row>
           <xdr:rowOff>0</xdr:rowOff>
         </xdr:to>
@@ -4590,7 +4590,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4620,9 +4620,9 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>942975</xdr:colOff>
+          <xdr:colOff>946150</xdr:colOff>
           <xdr:row>80</xdr:row>
-          <xdr:rowOff>66675</xdr:rowOff>
+          <xdr:rowOff>69850</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>6</xdr:col>
@@ -4672,7 +4672,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4708,9 +4708,9 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>638175</xdr:colOff>
+          <xdr:colOff>641350</xdr:colOff>
           <xdr:row>40</xdr:row>
-          <xdr:rowOff>276225</xdr:rowOff>
+          <xdr:rowOff>279400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4754,7 +4754,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4792,7 +4792,7 @@
           <xdr:col>3</xdr:col>
           <xdr:colOff>1181100</xdr:colOff>
           <xdr:row>40</xdr:row>
-          <xdr:rowOff>276225</xdr:rowOff>
+          <xdr:rowOff>279400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4836,7 +4836,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4872,9 +4872,9 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
-          <xdr:colOff>104775</xdr:colOff>
+          <xdr:colOff>107950</xdr:colOff>
           <xdr:row>40</xdr:row>
-          <xdr:rowOff>276225</xdr:rowOff>
+          <xdr:rowOff>279400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -4918,7 +4918,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -4956,7 +4956,7 @@
           <xdr:col>6</xdr:col>
           <xdr:colOff>381000</xdr:colOff>
           <xdr:row>40</xdr:row>
-          <xdr:rowOff>276225</xdr:rowOff>
+          <xdr:rowOff>279400</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5000,7 +5000,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -5032,7 +5032,7 @@
           <xdr:col>5</xdr:col>
           <xdr:colOff>304800</xdr:colOff>
           <xdr:row>61</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>31750</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>5</xdr:col>
@@ -5096,7 +5096,7 @@
           <xdr:col>6</xdr:col>
           <xdr:colOff>76200</xdr:colOff>
           <xdr:row>61</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>31750</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>6</xdr:col>
@@ -5158,13 +5158,13 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>7</xdr:col>
-          <xdr:colOff>314325</xdr:colOff>
+          <xdr:colOff>317500</xdr:colOff>
           <xdr:row>61</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>31750</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>7</xdr:col>
-          <xdr:colOff>600075</xdr:colOff>
+          <xdr:colOff>603250</xdr:colOff>
           <xdr:row>61</xdr:row>
           <xdr:rowOff>247650</xdr:rowOff>
         </xdr:to>
@@ -5222,9 +5222,9 @@
       <xdr:twoCellAnchor editAs="oneCell">
         <xdr:from>
           <xdr:col>7</xdr:col>
-          <xdr:colOff>1419225</xdr:colOff>
+          <xdr:colOff>1422400</xdr:colOff>
           <xdr:row>61</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>31750</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>8</xdr:col>
@@ -5288,7 +5288,7 @@
           <xdr:col>9</xdr:col>
           <xdr:colOff>0</xdr:colOff>
           <xdr:row>61</xdr:row>
-          <xdr:rowOff>28575</xdr:rowOff>
+          <xdr:rowOff>31750</xdr:rowOff>
         </xdr:from>
         <xdr:to>
           <xdr:col>9</xdr:col>
@@ -5356,9 +5356,9 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>638175</xdr:colOff>
+          <xdr:colOff>641350</xdr:colOff>
           <xdr:row>39</xdr:row>
-          <xdr:rowOff>257175</xdr:rowOff>
+          <xdr:rowOff>260350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5402,7 +5402,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -5438,9 +5438,9 @@
         </xdr:from>
         <xdr:to>
           <xdr:col>3</xdr:col>
-          <xdr:colOff>1362075</xdr:colOff>
+          <xdr:colOff>1365250</xdr:colOff>
           <xdr:row>39</xdr:row>
-          <xdr:rowOff>257175</xdr:rowOff>
+          <xdr:rowOff>260350</xdr:rowOff>
         </xdr:to>
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
@@ -5484,7 +5484,7 @@
             </a:extLst>
           </xdr:spPr>
           <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+            <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr algn="l" rtl="0">
@@ -5537,10 +5537,10 @@
           </xdr:nvGrpSpPr>
           <xdr:grpSpPr>
             <a:xfrm>
-              <a:off x="2943225" y="3743325"/>
-              <a:ext cx="1466850" cy="209550"/>
-              <a:chOff x="2266949" y="4686300"/>
-              <a:chExt cx="1685926" cy="209550"/>
+              <a:off x="3070225" y="3644900"/>
+              <a:ext cx="1524000" cy="209550"/>
+              <a:chOff x="2266950" y="4686300"/>
+              <a:chExt cx="1685925" cy="209550"/>
             </a:xfrm>
           </xdr:grpSpPr>
           <xdr:sp macro="" textlink="">
@@ -5559,7 +5559,7 @@
             </xdr:nvSpPr>
             <xdr:spPr bwMode="auto">
               <a:xfrm>
-                <a:off x="2266949" y="4686300"/>
+                <a:off x="2266950" y="4686300"/>
                 <a:ext cx="781050" cy="209550"/>
               </a:xfrm>
               <a:prstGeom prst="rect">
@@ -5585,7 +5585,7 @@
               </a:extLst>
             </xdr:spPr>
             <xdr:txBody>
-              <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+              <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr algn="l" rtl="0">
@@ -5647,7 +5647,7 @@
               </a:extLst>
             </xdr:spPr>
             <xdr:txBody>
-              <a:bodyPr vertOverflow="clip" wrap="square" lIns="27432" tIns="18288" rIns="0" bIns="18288" anchor="ctr" upright="1"/>
+              <a:bodyPr vertOverflow="clip" wrap="square" lIns="36576" tIns="22860" rIns="0" bIns="22860" anchor="ctr" upright="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr algn="l" rtl="0">
@@ -12845,7 +12845,7 @@
       <xdr:grpSpPr>
         <a:xfrm>
           <a:off x="419100" y="495300"/>
-          <a:ext cx="2452352" cy="1471142"/>
+          <a:ext cx="2585702" cy="1448917"/>
           <a:chOff x="4591734" y="1323376"/>
           <a:chExt cx="2252327" cy="1471142"/>
         </a:xfrm>
@@ -15117,41 +15117,41 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AP128"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="2.85546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="37.42578125" style="2" customWidth="1"/>
-    <col min="3" max="3" width="18.5703125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="21.42578125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="5.7109375" style="2" customWidth="1"/>
-    <col min="6" max="9" width="20.7109375" style="2" customWidth="1"/>
-    <col min="10" max="10" width="20.7109375" style="94" customWidth="1"/>
+    <col min="1" max="1" width="2.81640625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="37.453125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="18.54296875" style="2" customWidth="1"/>
+    <col min="4" max="4" width="21.453125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="5.7265625" style="2" customWidth="1"/>
+    <col min="6" max="9" width="20.7265625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="20.7265625" style="94" customWidth="1"/>
     <col min="11" max="11" width="5" style="94" customWidth="1"/>
-    <col min="12" max="12" width="11.7109375" style="94" customWidth="1"/>
-    <col min="13" max="15" width="10.85546875" style="94" customWidth="1"/>
-    <col min="16" max="21" width="10.85546875" style="2" customWidth="1"/>
-    <col min="22" max="25" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="27" max="28" width="9.140625" style="2"/>
-    <col min="29" max="32" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="9.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="9.140625" style="15"/>
-    <col min="35" max="35" width="9.140625" style="6"/>
-    <col min="36" max="36" width="9.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="9.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="38" max="39" width="9.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="9.28515625" style="6" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="9.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="9.140625" style="6"/>
-    <col min="43" max="16384" width="9.140625" style="2"/>
+    <col min="12" max="12" width="11.7265625" style="94" customWidth="1"/>
+    <col min="13" max="15" width="10.81640625" style="94" customWidth="1"/>
+    <col min="16" max="21" width="10.81640625" style="2" customWidth="1"/>
+    <col min="22" max="25" width="10.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="9.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="27" max="28" width="9.1796875" style="2"/>
+    <col min="29" max="32" width="10.54296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="9.453125" style="2" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="9.1796875" style="15"/>
+    <col min="35" max="35" width="9.1796875" style="6"/>
+    <col min="36" max="36" width="9.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="9.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="38" max="39" width="9.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="9.26953125" style="6" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="9.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="9.1796875" style="6"/>
+    <col min="43" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:42" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:42" x14ac:dyDescent="0.35">
       <c r="H1" s="92" t="s">
         <v>16</v>
       </c>
       <c r="I1" s="93">
-        <v>45884</v>
+        <v>46273</v>
       </c>
       <c r="P1" s="94"/>
       <c r="Q1" s="94"/>
@@ -15169,7 +15169,7 @@
       <c r="AO1" s="4"/>
       <c r="AP1" s="4"/>
     </row>
-    <row r="2" spans="1:42" ht="26.25" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:42" ht="26" x14ac:dyDescent="0.35">
       <c r="B2" s="291" t="s">
         <v>37</v>
       </c>
@@ -15183,7 +15183,7 @@
       <c r="U2" s="94"/>
       <c r="AI2" s="5"/>
     </row>
-    <row r="3" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="95" t="s">
         <v>38</v>
       </c>
@@ -15197,7 +15197,7 @@
       <c r="U3" s="94"/>
       <c r="AI3" s="5"/>
     </row>
-    <row r="4" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="95" t="s">
         <v>39</v>
       </c>
@@ -15211,7 +15211,7 @@
       <c r="U4" s="94"/>
       <c r="AI4" s="5"/>
     </row>
-    <row r="5" spans="1:42" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:42" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B5" s="96" t="s">
         <v>40</v>
       </c>
@@ -15225,7 +15225,7 @@
       <c r="U5" s="94"/>
       <c r="AI5" s="5"/>
     </row>
-    <row r="6" spans="1:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="65" t="s">
         <v>41</v>
       </c>
@@ -15252,7 +15252,7 @@
       <c r="AO6" s="6"/>
       <c r="AP6" s="6"/>
     </row>
-    <row r="7" spans="1:42" s="156" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:42" s="156" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B7" s="153" t="s">
         <v>278</v>
       </c>
@@ -15280,7 +15280,7 @@
       <c r="AO7" s="231"/>
       <c r="AP7" s="231"/>
     </row>
-    <row r="8" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:42" x14ac:dyDescent="0.35">
       <c r="C8" s="97" t="s">
         <v>240</v>
       </c>
@@ -15292,7 +15292,7 @@
       <c r="T8" s="94"/>
       <c r="U8" s="94"/>
     </row>
-    <row r="9" spans="1:42" ht="16.5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.35">
       <c r="C9" s="97"/>
       <c r="D9" s="97"/>
       <c r="P9" s="94"/>
@@ -15303,9 +15303,9 @@
       <c r="U9" s="94"/>
       <c r="AI9" s="69"/>
     </row>
-    <row r="10" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="68" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C10" s="97"/>
       <c r="D10" s="97"/>
@@ -15317,7 +15317,7 @@
       <c r="U10" s="94"/>
       <c r="AI10" s="71"/>
     </row>
-    <row r="11" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="99" t="s">
         <v>279</v>
       </c>
@@ -15330,7 +15330,7 @@
       <c r="T11" s="94"/>
       <c r="U11" s="94"/>
     </row>
-    <row r="12" spans="1:42" ht="17.25" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:42" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="100"/>
       <c r="C12" s="100"/>
       <c r="D12" s="100"/>
@@ -15347,7 +15347,7 @@
       <c r="U12" s="94"/>
       <c r="AI12" s="74"/>
     </row>
-    <row r="13" spans="1:42" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:42" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="170"/>
       <c r="B13" s="244" t="s">
         <v>267</v>
@@ -15372,19 +15372,19 @@
       <c r="AN13" s="75"/>
       <c r="AO13" s="75"/>
     </row>
-    <row r="14" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="170"/>
       <c r="B14" s="248" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="304"/>
-      <c r="D14" s="304"/>
+      <c r="C14" s="306"/>
+      <c r="D14" s="306"/>
       <c r="E14" s="170"/>
       <c r="F14" s="248" t="s">
         <v>272</v>
       </c>
-      <c r="G14" s="297"/>
-      <c r="H14" s="297"/>
+      <c r="G14" s="300"/>
+      <c r="H14" s="300"/>
       <c r="I14" s="272"/>
       <c r="P14" s="94"/>
       <c r="Q14" s="94"/>
@@ -15394,7 +15394,7 @@
       <c r="U14" s="94"/>
       <c r="AI14" s="15"/>
     </row>
-    <row r="15" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="170"/>
       <c r="B15" s="269" t="s">
         <v>44</v>
@@ -15405,8 +15405,8 @@
       <c r="F15" s="248" t="s">
         <v>263</v>
       </c>
-      <c r="G15" s="305"/>
-      <c r="H15" s="306"/>
+      <c r="G15" s="307"/>
+      <c r="H15" s="308"/>
       <c r="I15" s="272"/>
       <c r="P15" s="94"/>
       <c r="Q15" s="94"/>
@@ -15416,21 +15416,21 @@
       <c r="U15" s="94"/>
       <c r="AI15" s="15"/>
     </row>
-    <row r="16" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A16" s="170"/>
       <c r="B16" s="248" t="s">
         <v>45</v>
       </c>
-      <c r="C16" s="307"/>
-      <c r="D16" s="307"/>
+      <c r="C16" s="309"/>
+      <c r="D16" s="309"/>
       <c r="E16" s="170"/>
       <c r="F16" s="250" t="s">
         <v>264</v>
       </c>
-      <c r="G16" s="294" t="s">
+      <c r="G16" s="315" t="s">
         <v>269</v>
       </c>
-      <c r="H16" s="295"/>
+      <c r="H16" s="316"/>
       <c r="I16" s="272"/>
       <c r="K16" s="98"/>
       <c r="L16" s="98"/>
@@ -15450,21 +15450,21 @@
       <c r="AN16" s="79"/>
       <c r="AO16" s="79"/>
     </row>
-    <row r="17" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="170"/>
       <c r="B17" s="250" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="308"/>
-      <c r="D17" s="308"/>
+      <c r="C17" s="310"/>
+      <c r="D17" s="310"/>
       <c r="E17" s="170"/>
       <c r="F17" s="250" t="s">
         <v>265</v>
       </c>
-      <c r="G17" s="294" t="s">
+      <c r="G17" s="315" t="s">
         <v>270</v>
       </c>
-      <c r="H17" s="295"/>
+      <c r="H17" s="316"/>
       <c r="I17" s="272"/>
       <c r="J17" s="86"/>
       <c r="K17" s="98"/>
@@ -15485,21 +15485,21 @@
       <c r="AN17" s="80"/>
       <c r="AO17" s="80"/>
     </row>
-    <row r="18" spans="1:41" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:41" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="170"/>
       <c r="B18" s="273" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="309"/>
-      <c r="D18" s="309"/>
+      <c r="C18" s="311"/>
+      <c r="D18" s="311"/>
       <c r="E18" s="270"/>
       <c r="F18" s="251" t="s">
         <v>266</v>
       </c>
-      <c r="G18" s="296" t="s">
+      <c r="G18" s="317" t="s">
         <v>271</v>
       </c>
-      <c r="H18" s="296"/>
+      <c r="H18" s="317"/>
       <c r="I18" s="274"/>
       <c r="J18" s="86"/>
       <c r="K18" s="98"/>
@@ -15520,7 +15520,7 @@
       <c r="AN18" s="80"/>
       <c r="AO18" s="80"/>
     </row>
-    <row r="19" spans="1:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:41" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B19" s="100"/>
       <c r="C19" s="100"/>
       <c r="D19" s="102"/>
@@ -15543,7 +15543,7 @@
       <c r="AN19" s="81"/>
       <c r="AO19" s="81"/>
     </row>
-    <row r="20" spans="1:41" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:41" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="244" t="s">
         <v>268</v>
       </c>
@@ -15568,18 +15568,18 @@
       <c r="AN20" s="81"/>
       <c r="AO20" s="81"/>
     </row>
-    <row r="21" spans="1:41" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:41" ht="48.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="170"/>
       <c r="B21" s="248" t="s">
         <v>47</v>
       </c>
-      <c r="C21" s="298"/>
-      <c r="D21" s="298"/>
-      <c r="E21" s="298"/>
-      <c r="F21" s="298"/>
-      <c r="G21" s="298"/>
-      <c r="H21" s="298"/>
-      <c r="I21" s="299"/>
+      <c r="C21" s="301"/>
+      <c r="D21" s="301"/>
+      <c r="E21" s="301"/>
+      <c r="F21" s="301"/>
+      <c r="G21" s="301"/>
+      <c r="H21" s="301"/>
+      <c r="I21" s="302"/>
       <c r="P21" s="94"/>
       <c r="Q21" s="94"/>
       <c r="R21" s="94"/>
@@ -15594,18 +15594,18 @@
       <c r="AN21" s="81"/>
       <c r="AO21" s="81"/>
     </row>
-    <row r="22" spans="1:41" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:41" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="170"/>
       <c r="B22" s="248" t="s">
         <v>254</v>
       </c>
-      <c r="C22" s="298"/>
-      <c r="D22" s="298"/>
-      <c r="E22" s="298"/>
-      <c r="F22" s="298"/>
-      <c r="G22" s="298"/>
-      <c r="H22" s="298"/>
-      <c r="I22" s="299"/>
+      <c r="C22" s="301"/>
+      <c r="D22" s="301"/>
+      <c r="E22" s="301"/>
+      <c r="F22" s="301"/>
+      <c r="G22" s="301"/>
+      <c r="H22" s="301"/>
+      <c r="I22" s="302"/>
       <c r="J22" s="98"/>
       <c r="N22" s="171"/>
       <c r="O22" s="171"/>
@@ -15629,18 +15629,18 @@
       <c r="AN22" s="89"/>
       <c r="AO22" s="89"/>
     </row>
-    <row r="23" spans="1:41" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:41" ht="28.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="170"/>
       <c r="B23" s="248" t="s">
         <v>281</v>
       </c>
-      <c r="C23" s="298"/>
-      <c r="D23" s="298"/>
-      <c r="E23" s="298"/>
-      <c r="F23" s="298"/>
-      <c r="G23" s="298"/>
-      <c r="H23" s="298"/>
-      <c r="I23" s="299"/>
+      <c r="C23" s="301"/>
+      <c r="D23" s="301"/>
+      <c r="E23" s="301"/>
+      <c r="F23" s="301"/>
+      <c r="G23" s="301"/>
+      <c r="H23" s="301"/>
+      <c r="I23" s="302"/>
       <c r="J23" s="98"/>
       <c r="N23" s="171"/>
       <c r="O23" s="171"/>
@@ -15664,18 +15664,18 @@
       <c r="AN23" s="89"/>
       <c r="AO23" s="89"/>
     </row>
-    <row r="24" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="170"/>
-      <c r="B24" s="300" t="s">
+      <c r="B24" s="303" t="s">
         <v>239</v>
       </c>
-      <c r="C24" s="301"/>
-      <c r="D24" s="301"/>
-      <c r="E24" s="301"/>
-      <c r="F24" s="301"/>
-      <c r="G24" s="301"/>
-      <c r="H24" s="301"/>
-      <c r="I24" s="302"/>
+      <c r="C24" s="304"/>
+      <c r="D24" s="304"/>
+      <c r="E24" s="304"/>
+      <c r="F24" s="304"/>
+      <c r="G24" s="304"/>
+      <c r="H24" s="304"/>
+      <c r="I24" s="305"/>
       <c r="P24" s="94"/>
       <c r="Q24" s="94"/>
       <c r="R24" s="94"/>
@@ -15690,15 +15690,15 @@
       <c r="AN24" s="81"/>
       <c r="AO24" s="81"/>
     </row>
-    <row r="25" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B25" s="300"/>
-      <c r="C25" s="301"/>
-      <c r="D25" s="301"/>
-      <c r="E25" s="301"/>
-      <c r="F25" s="301"/>
-      <c r="G25" s="301"/>
-      <c r="H25" s="301"/>
-      <c r="I25" s="302"/>
+    <row r="25" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="303"/>
+      <c r="C25" s="304"/>
+      <c r="D25" s="304"/>
+      <c r="E25" s="304"/>
+      <c r="F25" s="304"/>
+      <c r="G25" s="304"/>
+      <c r="H25" s="304"/>
+      <c r="I25" s="305"/>
       <c r="P25" s="94"/>
       <c r="Q25" s="94"/>
       <c r="R25" s="94"/>
@@ -15713,19 +15713,19 @@
       <c r="AN25" s="81"/>
       <c r="AO25" s="81"/>
     </row>
-    <row r="26" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="279" t="s">
         <v>257</v>
       </c>
       <c r="C26" s="278">
         <v>1</v>
       </c>
-      <c r="D26" s="292">
+      <c r="D26" s="313">
         <f>ROUNDUP((2+($C26*$C27*140)/60),0)</f>
         <v>5</v>
       </c>
-      <c r="E26" s="293" t="s">
-        <v>293</v>
+      <c r="E26" s="314" t="s">
+        <v>292</v>
       </c>
       <c r="F26" s="235"/>
       <c r="G26" s="235"/>
@@ -15745,15 +15745,15 @@
       <c r="AN26" s="81"/>
       <c r="AO26" s="81"/>
     </row>
-    <row r="27" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="281" t="s">
         <v>275</v>
       </c>
       <c r="C27" s="243">
         <v>1</v>
       </c>
-      <c r="D27" s="292"/>
-      <c r="E27" s="293"/>
+      <c r="D27" s="313"/>
+      <c r="E27" s="314"/>
       <c r="F27" s="235"/>
       <c r="G27" s="235"/>
       <c r="H27" s="235"/>
@@ -15772,7 +15772,7 @@
       <c r="AN27" s="81"/>
       <c r="AO27" s="81"/>
     </row>
-    <row r="28" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="282" t="s">
         <v>262</v>
       </c>
@@ -15784,7 +15784,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="240" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F28" s="235"/>
       <c r="G28" s="235"/>
@@ -15804,7 +15804,7 @@
       <c r="AN28" s="81"/>
       <c r="AO28" s="81"/>
     </row>
-    <row r="29" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="283" t="s">
         <v>67</v>
       </c>
@@ -15816,7 +15816,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="240" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F29" s="235"/>
       <c r="G29" s="235"/>
@@ -15836,9 +15836,9 @@
       <c r="AN29" s="81"/>
       <c r="AO29" s="81"/>
     </row>
-    <row r="30" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="284" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C30" s="275">
         <f>C26*C27+C28+C29</f>
@@ -15849,7 +15849,7 @@
         <v>5</v>
       </c>
       <c r="E30" s="277" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="F30" s="235"/>
       <c r="G30" s="235"/>
@@ -15869,14 +15869,14 @@
       <c r="AN30" s="81"/>
       <c r="AO30" s="81"/>
     </row>
-    <row r="31" spans="1:41" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:41" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B31" s="285" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C31" s="286"/>
       <c r="D31" s="287">
         <f>P79+D30*P78</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="E31" s="288"/>
       <c r="F31" s="289"/>
@@ -15897,7 +15897,7 @@
       <c r="AN31" s="81"/>
       <c r="AO31" s="81"/>
     </row>
-    <row r="32" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:41" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C32" s="235"/>
       <c r="D32" s="235"/>
       <c r="E32" s="235"/>
@@ -15919,17 +15919,17 @@
       <c r="AN32" s="81"/>
       <c r="AO32" s="81"/>
     </row>
-    <row r="33" spans="2:41" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B33" s="314" t="s">
-        <v>296</v>
-      </c>
-      <c r="C33" s="314"/>
-      <c r="D33" s="314"/>
-      <c r="E33" s="314"/>
-      <c r="F33" s="314"/>
-      <c r="G33" s="314"/>
-      <c r="H33" s="314"/>
-      <c r="I33" s="314"/>
+    <row r="33" spans="2:41" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B33" s="299" t="s">
+        <v>295</v>
+      </c>
+      <c r="C33" s="299"/>
+      <c r="D33" s="299"/>
+      <c r="E33" s="299"/>
+      <c r="F33" s="299"/>
+      <c r="G33" s="299"/>
+      <c r="H33" s="299"/>
+      <c r="I33" s="299"/>
       <c r="P33" s="94"/>
       <c r="Q33" s="94"/>
       <c r="R33" s="94"/>
@@ -15944,7 +15944,7 @@
       <c r="AN33" s="81"/>
       <c r="AO33" s="81"/>
     </row>
-    <row r="34" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="65" t="s">
         <v>48</v>
       </c>
@@ -15967,7 +15967,7 @@
       <c r="AN34" s="81"/>
       <c r="AO34" s="81"/>
     </row>
-    <row r="35" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="68" t="s">
         <v>50</v>
       </c>
@@ -15990,16 +15990,16 @@
       <c r="AN35" s="81"/>
       <c r="AO35" s="81"/>
     </row>
-    <row r="36" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="65" t="s">
         <v>58</v>
       </c>
       <c r="C36" s="65"/>
-      <c r="D36" s="311"/>
-      <c r="E36" s="311"/>
-      <c r="F36" s="311"/>
-      <c r="G36" s="311"/>
-      <c r="H36" s="311"/>
+      <c r="D36" s="312"/>
+      <c r="E36" s="312"/>
+      <c r="F36" s="312"/>
+      <c r="G36" s="312"/>
+      <c r="H36" s="312"/>
       <c r="P36" s="94"/>
       <c r="Q36" s="94"/>
       <c r="R36" s="94"/>
@@ -16015,7 +16015,7 @@
       <c r="AN36" s="81"/>
       <c r="AO36" s="81"/>
     </row>
-    <row r="37" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="65" t="s">
         <v>51</v>
       </c>
@@ -16046,7 +16046,7 @@
       <c r="AN37" s="81"/>
       <c r="AO37" s="81"/>
     </row>
-    <row r="38" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="65" t="s">
         <v>54</v>
       </c>
@@ -16077,16 +16077,16 @@
       <c r="AN38" s="81"/>
       <c r="AO38" s="81"/>
     </row>
-    <row r="39" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="65" t="s">
         <v>57</v>
       </c>
       <c r="C39" s="65"/>
-      <c r="D39" s="303"/>
-      <c r="E39" s="303"/>
-      <c r="F39" s="303"/>
-      <c r="G39" s="303"/>
-      <c r="H39" s="303"/>
+      <c r="D39" s="297"/>
+      <c r="E39" s="297"/>
+      <c r="F39" s="297"/>
+      <c r="G39" s="297"/>
+      <c r="H39" s="297"/>
       <c r="P39" s="94"/>
       <c r="Q39" s="94"/>
       <c r="R39" s="94"/>
@@ -16102,16 +16102,16 @@
       <c r="AN39" s="81"/>
       <c r="AO39" s="81"/>
     </row>
-    <row r="40" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="65" t="s">
         <v>59</v>
       </c>
       <c r="C40" s="65"/>
-      <c r="D40" s="312"/>
-      <c r="E40" s="312"/>
-      <c r="F40" s="312"/>
-      <c r="G40" s="312"/>
-      <c r="H40" s="312"/>
+      <c r="D40" s="296"/>
+      <c r="E40" s="296"/>
+      <c r="F40" s="296"/>
+      <c r="G40" s="296"/>
+      <c r="H40" s="296"/>
       <c r="P40" s="94"/>
       <c r="Q40" s="94"/>
       <c r="R40" s="94"/>
@@ -16127,7 +16127,7 @@
       <c r="AN40" s="81"/>
       <c r="AO40" s="81"/>
     </row>
-    <row r="41" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="65" t="s">
         <v>60</v>
       </c>
@@ -16152,16 +16152,16 @@
       <c r="AN41" s="81"/>
       <c r="AO41" s="81"/>
     </row>
-    <row r="42" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C42" s="65"/>
-      <c r="D42" s="303"/>
-      <c r="E42" s="303"/>
-      <c r="F42" s="303"/>
-      <c r="G42" s="303"/>
-      <c r="H42" s="303"/>
+      <c r="D42" s="297"/>
+      <c r="E42" s="297"/>
+      <c r="F42" s="297"/>
+      <c r="G42" s="297"/>
+      <c r="H42" s="297"/>
       <c r="P42" s="94"/>
       <c r="Q42" s="94"/>
       <c r="R42" s="94"/>
@@ -16177,16 +16177,16 @@
       <c r="AN42" s="81"/>
       <c r="AO42" s="81"/>
     </row>
-    <row r="43" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="65" t="s">
         <v>62</v>
       </c>
       <c r="C43" s="65"/>
-      <c r="D43" s="313"/>
-      <c r="E43" s="313"/>
-      <c r="F43" s="313"/>
-      <c r="G43" s="313"/>
-      <c r="H43" s="313"/>
+      <c r="D43" s="298"/>
+      <c r="E43" s="298"/>
+      <c r="F43" s="298"/>
+      <c r="G43" s="298"/>
+      <c r="H43" s="298"/>
       <c r="P43" s="94"/>
       <c r="Q43" s="94"/>
       <c r="R43" s="94"/>
@@ -16202,7 +16202,7 @@
       <c r="AN43" s="81"/>
       <c r="AO43" s="81"/>
     </row>
-    <row r="44" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="97" t="s">
         <v>282</v>
       </c>
@@ -16227,16 +16227,16 @@
       <c r="AN44" s="81"/>
       <c r="AO44" s="81"/>
     </row>
-    <row r="45" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="65" t="s">
         <v>280</v>
       </c>
       <c r="C45" s="65"/>
-      <c r="D45" s="303"/>
-      <c r="E45" s="303"/>
-      <c r="F45" s="303"/>
-      <c r="G45" s="303"/>
-      <c r="H45" s="303"/>
+      <c r="D45" s="297"/>
+      <c r="E45" s="297"/>
+      <c r="F45" s="297"/>
+      <c r="G45" s="297"/>
+      <c r="H45" s="297"/>
       <c r="P45" s="94"/>
       <c r="Q45" s="94"/>
       <c r="R45" s="94"/>
@@ -16252,7 +16252,7 @@
       <c r="AN45" s="81"/>
       <c r="AO45" s="81"/>
     </row>
-    <row r="46" spans="2:41" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="2:41" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B46" s="102"/>
       <c r="C46" s="102"/>
       <c r="D46" s="102"/>
@@ -16277,7 +16277,7 @@
       <c r="AN46" s="81"/>
       <c r="AO46" s="81"/>
     </row>
-    <row r="47" spans="2:41" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:41" ht="33.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="66" t="s">
         <v>283</v>
       </c>
@@ -16297,7 +16297,7 @@
       <c r="AN47" s="81"/>
       <c r="AO47" s="81"/>
     </row>
-    <row r="48" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="67" t="s">
         <v>63</v>
       </c>
@@ -16317,7 +16317,7 @@
       <c r="AN48" s="81"/>
       <c r="AO48" s="81"/>
     </row>
-    <row r="49" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B49" s="65" t="s">
         <v>273</v>
       </c>
@@ -16341,7 +16341,7 @@
       <c r="AN49" s="81"/>
       <c r="AO49" s="81"/>
     </row>
-    <row r="50" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="65" t="s">
         <v>274</v>
       </c>
@@ -16365,7 +16365,7 @@
       <c r="AN50" s="81"/>
       <c r="AO50" s="81"/>
     </row>
-    <row r="51" spans="2:42" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="2:42" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="P51" s="94"/>
       <c r="Q51" s="94"/>
       <c r="R51" s="94"/>
@@ -16380,7 +16380,7 @@
       <c r="AN51" s="81"/>
       <c r="AO51" s="81"/>
     </row>
-    <row r="52" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="67" t="s">
         <v>65</v>
       </c>
@@ -16394,7 +16394,7 @@
       <c r="AM52" s="88"/>
       <c r="AO52" s="88"/>
     </row>
-    <row r="53" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B53" s="65" t="s">
         <v>17</v>
       </c>
@@ -16414,7 +16414,7 @@
       <c r="AN53" s="79"/>
       <c r="AO53" s="79"/>
     </row>
-    <row r="54" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="65" t="s">
         <v>244</v>
       </c>
@@ -16434,16 +16434,16 @@
       <c r="AN54" s="80"/>
       <c r="AO54" s="80"/>
     </row>
-    <row r="55" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="65" t="s">
         <v>255</v>
       </c>
       <c r="C55" s="65"/>
       <c r="D55" s="65"/>
-      <c r="E55" s="310"/>
-      <c r="F55" s="310"/>
-      <c r="G55" s="310"/>
-      <c r="H55" s="310"/>
+      <c r="E55" s="292"/>
+      <c r="F55" s="292"/>
+      <c r="G55" s="292"/>
+      <c r="H55" s="292"/>
       <c r="P55" s="94"/>
       <c r="Q55" s="94"/>
       <c r="R55" s="94"/>
@@ -16458,7 +16458,7 @@
       <c r="AN55" s="80"/>
       <c r="AO55" s="80"/>
     </row>
-    <row r="56" spans="2:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="2:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="65" t="s">
         <v>256</v>
       </c>
@@ -16489,15 +16489,15 @@
       <c r="AO56" s="89"/>
       <c r="AP56" s="6"/>
     </row>
-    <row r="57" spans="2:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="2:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="70" t="s">
         <v>66</v>
       </c>
       <c r="D57" s="107"/>
-      <c r="E57" s="310"/>
-      <c r="F57" s="310"/>
-      <c r="G57" s="310"/>
-      <c r="H57" s="310"/>
+      <c r="E57" s="292"/>
+      <c r="F57" s="292"/>
+      <c r="G57" s="292"/>
+      <c r="H57" s="292"/>
       <c r="J57" s="98"/>
       <c r="K57" s="98"/>
       <c r="L57" s="98"/>
@@ -16520,7 +16520,7 @@
       <c r="AO57" s="89"/>
       <c r="AP57" s="6"/>
     </row>
-    <row r="58" spans="2:42" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:42" ht="33" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B58" s="108" t="s">
         <v>18</v>
       </c>
@@ -16544,7 +16544,7 @@
       <c r="AN58" s="89"/>
       <c r="AO58" s="89"/>
     </row>
-    <row r="59" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="65" t="s">
         <v>19</v>
       </c>
@@ -16576,7 +16576,7 @@
       <c r="AN59" s="89"/>
       <c r="AO59" s="89"/>
     </row>
-    <row r="60" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="65" t="s">
         <v>21</v>
       </c>
@@ -16609,7 +16609,7 @@
       <c r="AN60" s="89"/>
       <c r="AO60" s="89"/>
     </row>
-    <row r="61" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C61" s="65"/>
       <c r="D61" s="107"/>
       <c r="E61" s="76"/>
@@ -16630,7 +16630,7 @@
       <c r="AN61" s="89"/>
       <c r="AO61" s="89"/>
     </row>
-    <row r="62" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="133" t="s">
         <v>22</v>
       </c>
@@ -16664,7 +16664,7 @@
       <c r="AN62" s="89"/>
       <c r="AO62" s="89"/>
     </row>
-    <row r="63" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="2:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="77" t="s">
         <v>28</v>
       </c>
@@ -16697,7 +16697,7 @@
       <c r="AN63" s="89"/>
       <c r="AO63" s="89"/>
     </row>
-    <row r="64" spans="2:42" s="47" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="2:42" s="47" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B64" s="143" t="s">
         <v>29</v>
       </c>
@@ -16732,7 +16732,7 @@
       <c r="AO64" s="150"/>
       <c r="AP64" s="151"/>
     </row>
-    <row r="65" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B65" s="77" t="s">
         <v>30</v>
       </c>
@@ -16765,7 +16765,7 @@
       <c r="AN65" s="89"/>
       <c r="AO65" s="89"/>
     </row>
-    <row r="66" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B66" s="77" t="s">
         <v>31</v>
       </c>
@@ -16798,7 +16798,7 @@
       <c r="AN66" s="89"/>
       <c r="AO66" s="89"/>
     </row>
-    <row r="67" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B67" s="77" t="s">
         <v>32</v>
       </c>
@@ -16821,10 +16821,10 @@
       </c>
       <c r="L67" s="2"/>
       <c r="M67" s="2"/>
-      <c r="O67" s="310"/>
-      <c r="P67" s="310"/>
-      <c r="Q67" s="310"/>
-      <c r="R67" s="310"/>
+      <c r="O67" s="292"/>
+      <c r="P67" s="292"/>
+      <c r="Q67" s="292"/>
+      <c r="R67" s="292"/>
       <c r="AI67" s="80"/>
       <c r="AJ67" s="89"/>
       <c r="AK67" s="89"/>
@@ -16833,7 +16833,7 @@
       <c r="AN67" s="89"/>
       <c r="AO67" s="89"/>
     </row>
-    <row r="68" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="77" t="s">
         <v>33</v>
       </c>
@@ -16878,7 +16878,7 @@
       <c r="AN68" s="89"/>
       <c r="AO68" s="89"/>
     </row>
-    <row r="69" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B69" s="83" t="s">
         <v>35</v>
       </c>
@@ -16923,7 +16923,7 @@
       <c r="AN69" s="89"/>
       <c r="AO69" s="89"/>
     </row>
-    <row r="70" spans="1:42" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:42" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="127"/>
       <c r="C70" s="128"/>
       <c r="D70" s="129" t="s">
@@ -16963,7 +16963,7 @@
       <c r="AN70" s="89"/>
       <c r="AO70" s="89"/>
     </row>
-    <row r="71" spans="1:42" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:42" ht="25.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B71" s="65"/>
       <c r="C71" s="85"/>
       <c r="D71" s="129" t="s">
@@ -16972,23 +16972,23 @@
       <c r="E71" s="130"/>
       <c r="F71" s="197">
         <f>F$70*$P$78+$P$79</f>
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="G71" s="196">
         <f>G$70*$P$78+$P$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="H71" s="198">
         <f>H$70*$P$78+$P$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="I71" s="198">
         <f>I$70*$P$78+$P$79</f>
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="J71" s="199">
         <f>J$70*$P$78+$P$79</f>
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="K71" s="98"/>
       <c r="AI71" s="80"/>
@@ -16999,7 +16999,7 @@
       <c r="AN71" s="89"/>
       <c r="AO71" s="89"/>
     </row>
-    <row r="72" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B72" s="65"/>
       <c r="C72" s="85"/>
       <c r="D72" s="200" t="s">
@@ -17029,7 +17029,7 @@
       <c r="AN72" s="89"/>
       <c r="AO72" s="89"/>
     </row>
-    <row r="73" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B73" s="65"/>
       <c r="C73" s="85"/>
       <c r="D73" s="176" t="s">
@@ -17058,7 +17058,7 @@
       <c r="AN73" s="89"/>
       <c r="AO73" s="89"/>
     </row>
-    <row r="74" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B74" s="65"/>
       <c r="C74" s="85"/>
       <c r="D74" s="176" t="s">
@@ -17087,7 +17087,7 @@
       <c r="AN74" s="89"/>
       <c r="AO74" s="89"/>
     </row>
-    <row r="75" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B75" s="65"/>
       <c r="C75" s="85"/>
       <c r="D75" s="206" t="s">
@@ -17117,7 +17117,7 @@
       <c r="AN75" s="89"/>
       <c r="AO75" s="89"/>
     </row>
-    <row r="76" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B76" s="65"/>
       <c r="C76" s="85"/>
       <c r="E76" s="115"/>
@@ -17151,15 +17151,15 @@
       <c r="AN76" s="89"/>
       <c r="AO76" s="89"/>
     </row>
-    <row r="77" spans="1:42" s="85" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:42" s="85" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B77" s="68" t="s">
         <v>284</v>
       </c>
-      <c r="C77" s="303"/>
-      <c r="D77" s="303"/>
-      <c r="E77" s="303"/>
-      <c r="F77" s="303"/>
-      <c r="G77" s="303"/>
+      <c r="C77" s="297"/>
+      <c r="D77" s="297"/>
+      <c r="E77" s="297"/>
+      <c r="F77" s="297"/>
+      <c r="G77" s="297"/>
       <c r="K77" s="101"/>
       <c r="L77" s="101"/>
       <c r="M77" s="192"/>
@@ -17204,7 +17204,7 @@
       <c r="AO77" s="194"/>
       <c r="AP77" s="195"/>
     </row>
-    <row r="78" spans="1:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:42" s="65" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A78" s="2"/>
       <c r="C78" s="85"/>
       <c r="D78" s="85"/>
@@ -17221,27 +17221,27 @@
       </c>
       <c r="O78" s="222">
         <f>Rates!E31</f>
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="P78" s="222">
         <f>Rates!F31</f>
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="Q78" s="222">
         <f>Rates!G31</f>
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="R78" s="222">
         <f>Rates!H31</f>
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="S78" s="222">
         <f>Rates!I31</f>
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="T78" s="185">
         <f>Rates!J31</f>
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="AB78" s="186"/>
       <c r="AC78" s="187"/>
@@ -17259,7 +17259,7 @@
       <c r="AO78" s="190"/>
       <c r="AP78" s="191"/>
     </row>
-    <row r="79" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B79" s="67" t="s">
         <v>75</v>
       </c>
@@ -17304,15 +17304,15 @@
       <c r="AN79" s="80"/>
       <c r="AO79" s="80"/>
     </row>
-    <row r="80" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:42" ht="22.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B80" s="65" t="s">
         <v>78</v>
       </c>
       <c r="C80" s="72" t="s">
         <v>79</v>
       </c>
-      <c r="D80" s="315"/>
-      <c r="E80" s="315"/>
+      <c r="D80" s="293"/>
+      <c r="E80" s="293"/>
       <c r="F80" s="72" t="s">
         <v>80</v>
       </c>
@@ -17341,7 +17341,7 @@
       <c r="AN80" s="89"/>
       <c r="AO80" s="89"/>
     </row>
-    <row r="81" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="81" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B81" s="65" t="s">
         <v>81</v>
       </c>
@@ -17355,27 +17355,27 @@
       <c r="N81" s="225"/>
       <c r="O81" s="224">
         <f t="shared" ref="O81" si="3">$F$70*O$78+O$79</f>
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="P81" s="224">
         <f>$F$70*P$78+P$79</f>
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="Q81" s="224">
         <f>$F$70*Q$78+Q$79</f>
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="R81" s="224">
         <f>$F$70*R$78+R$79</f>
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="S81" s="224">
         <f>$F$70*S$78+S$79</f>
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="T81" s="122">
         <f>$F$70*T$78+T$79</f>
-        <v>147</v>
+        <v>175</v>
       </c>
       <c r="AB81" s="116"/>
       <c r="AC81" s="117"/>
@@ -17391,13 +17391,13 @@
       <c r="AN81" s="89"/>
       <c r="AO81" s="89"/>
     </row>
-    <row r="82" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="82" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B82" s="65"/>
       <c r="C82" s="72" t="s">
         <v>79</v>
       </c>
-      <c r="D82" s="316"/>
-      <c r="E82" s="316"/>
+      <c r="D82" s="294"/>
+      <c r="E82" s="294"/>
       <c r="F82" s="72" t="s">
         <v>80</v>
       </c>
@@ -17408,27 +17408,27 @@
       <c r="N82" s="226"/>
       <c r="O82" s="227">
         <f t="shared" ref="O82" si="4">$G$70*O$78+O$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="P82" s="227">
         <f>$G$70*P$78+P$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="Q82" s="227">
         <f>$G$70*Q$78+Q$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="R82" s="227">
         <f>$G$70*R$78+R$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="S82" s="227">
         <f>$G$70*S$78+S$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="T82" s="124">
         <f>$G$70*T$78+T$79</f>
-        <v>177</v>
+        <v>212</v>
       </c>
       <c r="AB82" s="118"/>
       <c r="AC82" s="87"/>
@@ -17444,43 +17444,43 @@
       <c r="AN82" s="89"/>
       <c r="AO82" s="89"/>
     </row>
-    <row r="83" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B83" s="65" t="s">
         <v>83</v>
       </c>
       <c r="C83" s="65"/>
-      <c r="D83" s="317"/>
-      <c r="E83" s="317"/>
-      <c r="F83" s="317"/>
-      <c r="G83" s="317"/>
-      <c r="H83" s="317"/>
+      <c r="D83" s="295"/>
+      <c r="E83" s="295"/>
+      <c r="F83" s="295"/>
+      <c r="G83" s="295"/>
+      <c r="H83" s="295"/>
       <c r="M83" s="175" t="s">
         <v>25</v>
       </c>
       <c r="N83" s="225"/>
       <c r="O83" s="224">
         <f t="shared" ref="O83" si="5">$H$70*O$78+O$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="P83" s="224">
         <f>$H$70*P$78+P$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="Q83" s="224">
         <f>$H$70*Q$78+Q$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="R83" s="224">
         <f>$H$70*R$78+R$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="S83" s="224">
         <f>$H$70*S$78+S$79</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="T83" s="122">
         <f>$H$70*T$78+T$79</f>
-        <v>177</v>
+        <v>212</v>
       </c>
       <c r="AB83" s="118"/>
       <c r="AC83" s="87"/>
@@ -17496,7 +17496,7 @@
       <c r="AN83" s="89"/>
       <c r="AO83" s="89"/>
     </row>
-    <row r="84" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B84" s="65"/>
       <c r="C84" s="65"/>
       <c r="D84" s="65"/>
@@ -17506,27 +17506,27 @@
       <c r="N84" s="225"/>
       <c r="O84" s="224">
         <f t="shared" ref="O84" si="6">$I$70*O$78+O$79</f>
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="P84" s="224">
         <f>$I$70*P$78+P$79</f>
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="Q84" s="224">
         <f>$I$70*Q$78+Q$79</f>
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="R84" s="224">
         <f>$I$70*R$78+R$79</f>
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="S84" s="224">
         <f>$I$70*S$78+S$79</f>
-        <v>231</v>
+        <v>249</v>
       </c>
       <c r="T84" s="122">
         <f>$I$70*T$78+T$79</f>
-        <v>207</v>
+        <v>249</v>
       </c>
       <c r="AB84" s="118"/>
       <c r="AC84" s="87"/>
@@ -17542,7 +17542,7 @@
       <c r="AN84" s="89"/>
       <c r="AO84" s="89"/>
     </row>
-    <row r="85" spans="2:41" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="2:41" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B85" s="100"/>
       <c r="C85" s="102"/>
       <c r="D85" s="102"/>
@@ -17557,27 +17557,27 @@
       <c r="N85" s="225"/>
       <c r="O85" s="224">
         <f t="shared" ref="O85" si="7">$J$70*O$78+O$79</f>
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="P85" s="224">
         <f>$J$70*P$78+P$79</f>
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="Q85" s="224">
         <f>$J$70*Q$78+Q$79</f>
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="R85" s="224">
         <f>$J$70*R$78+R$79</f>
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="S85" s="224">
         <f>$J$70*S$78+S$79</f>
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="T85" s="122">
         <f>$J$70*T$78+T$79</f>
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="AB85" s="118"/>
       <c r="AC85" s="87"/>
@@ -17593,7 +17593,7 @@
       <c r="AN85" s="89"/>
       <c r="AO85" s="89"/>
     </row>
-    <row r="86" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B86" s="67"/>
       <c r="C86" s="65"/>
       <c r="D86" s="98"/>
@@ -17617,7 +17617,7 @@
       <c r="AN86" s="89"/>
       <c r="AO86" s="89"/>
     </row>
-    <row r="87" spans="2:41" x14ac:dyDescent="0.25">
+    <row r="87" spans="2:41" x14ac:dyDescent="0.35">
       <c r="B87" s="65"/>
       <c r="M87" s="206" t="s">
         <v>85</v>
@@ -17643,7 +17643,7 @@
       <c r="AN87" s="89"/>
       <c r="AO87" s="89"/>
     </row>
-    <row r="88" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B88" s="67" t="s">
         <v>285</v>
       </c>
@@ -17657,14 +17657,14 @@
       <c r="AN88" s="89"/>
       <c r="AO88" s="89"/>
     </row>
-    <row r="89" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="89" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B89" s="65"/>
       <c r="C89" s="65"/>
-      <c r="D89" s="312"/>
-      <c r="E89" s="312"/>
-      <c r="F89" s="312"/>
-      <c r="G89" s="312"/>
-      <c r="H89" s="312"/>
+      <c r="D89" s="296"/>
+      <c r="E89" s="296"/>
+      <c r="F89" s="296"/>
+      <c r="G89" s="296"/>
+      <c r="H89" s="296"/>
       <c r="N89" s="228"/>
       <c r="O89" s="228"/>
       <c r="AB89" s="116"/>
@@ -17681,7 +17681,7 @@
       <c r="AN89" s="89"/>
       <c r="AO89" s="89"/>
     </row>
-    <row r="90" spans="2:41" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="90" spans="2:41" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="236" t="s">
         <v>286</v>
       </c>
@@ -17711,7 +17711,7 @@
       <c r="AN90" s="89"/>
       <c r="AO90" s="89"/>
     </row>
-    <row r="91" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="91" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="M91" s="171"/>
       <c r="N91" s="171"/>
       <c r="O91" s="171"/>
@@ -17729,7 +17729,7 @@
       <c r="AN91" s="89"/>
       <c r="AO91" s="89"/>
     </row>
-    <row r="92" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="92" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB92" s="118"/>
       <c r="AC92" s="87"/>
       <c r="AD92" s="87"/>
@@ -17744,7 +17744,7 @@
       <c r="AN92" s="89"/>
       <c r="AO92" s="89"/>
     </row>
-    <row r="93" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="93" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AB93" s="118"/>
       <c r="AC93" s="87"/>
       <c r="AD93" s="87"/>
@@ -17759,7 +17759,7 @@
       <c r="AN93" s="89"/>
       <c r="AO93" s="89"/>
     </row>
-    <row r="94" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="94" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C94" s="65"/>
       <c r="D94" s="65"/>
       <c r="AI94" s="80"/>
@@ -17770,7 +17770,7 @@
       <c r="AN94" s="89"/>
       <c r="AO94" s="89"/>
     </row>
-    <row r="95" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="95" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI95" s="80"/>
       <c r="AJ95" s="89"/>
       <c r="AK95" s="89"/>
@@ -17779,7 +17779,7 @@
       <c r="AN95" s="89"/>
       <c r="AO95" s="89"/>
     </row>
-    <row r="96" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="96" spans="2:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI96" s="80"/>
       <c r="AJ96" s="89"/>
       <c r="AK96" s="89"/>
@@ -17788,7 +17788,7 @@
       <c r="AN96" s="89"/>
       <c r="AO96" s="89"/>
     </row>
-    <row r="97" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="97" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI97" s="80"/>
       <c r="AJ97" s="89"/>
       <c r="AK97" s="89"/>
@@ -17797,7 +17797,7 @@
       <c r="AN97" s="89"/>
       <c r="AO97" s="89"/>
     </row>
-    <row r="98" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="98" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI98" s="80"/>
       <c r="AJ98" s="89"/>
       <c r="AK98" s="89"/>
@@ -17806,7 +17806,7 @@
       <c r="AN98" s="89"/>
       <c r="AO98" s="89"/>
     </row>
-    <row r="99" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="99" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI99" s="80"/>
       <c r="AJ99" s="89"/>
       <c r="AK99" s="89"/>
@@ -17815,7 +17815,7 @@
       <c r="AN99" s="89"/>
       <c r="AO99" s="89"/>
     </row>
-    <row r="100" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="100" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI100" s="80"/>
       <c r="AJ100" s="89"/>
       <c r="AK100" s="89"/>
@@ -17824,8 +17824,8 @@
       <c r="AN100" s="89"/>
       <c r="AO100" s="89"/>
     </row>
-    <row r="101" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="101" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="102" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="AI102" s="78"/>
       <c r="AJ102" s="79"/>
       <c r="AK102" s="79"/>
@@ -17834,7 +17834,7 @@
       <c r="AN102" s="79"/>
       <c r="AO102" s="79"/>
     </row>
-    <row r="103" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="35:41" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI103" s="80"/>
       <c r="AJ103" s="80"/>
       <c r="AK103" s="80"/>
@@ -17843,7 +17843,7 @@
       <c r="AN103" s="80"/>
       <c r="AO103" s="80"/>
     </row>
-    <row r="104" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI104" s="80"/>
       <c r="AJ104" s="80"/>
       <c r="AK104" s="80"/>
@@ -17852,7 +17852,7 @@
       <c r="AN104" s="80"/>
       <c r="AO104" s="80"/>
     </row>
-    <row r="105" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI105" s="80"/>
       <c r="AJ105" s="89"/>
       <c r="AK105" s="89"/>
@@ -17861,7 +17861,7 @@
       <c r="AN105" s="89"/>
       <c r="AO105" s="89"/>
     </row>
-    <row r="106" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI106" s="80"/>
       <c r="AJ106" s="89"/>
       <c r="AK106" s="89"/>
@@ -17870,7 +17870,7 @@
       <c r="AN106" s="89"/>
       <c r="AO106" s="89"/>
     </row>
-    <row r="107" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="35:41" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="AI107" s="80"/>
       <c r="AJ107" s="89"/>
       <c r="AK107" s="89"/>
@@ -17879,7 +17879,7 @@
       <c r="AN107" s="89"/>
       <c r="AO107" s="89"/>
     </row>
-    <row r="108" spans="35:41" x14ac:dyDescent="0.25">
+    <row r="108" spans="35:41" x14ac:dyDescent="0.35">
       <c r="AI108" s="80"/>
       <c r="AJ108" s="89"/>
       <c r="AK108" s="89"/>
@@ -17888,7 +17888,7 @@
       <c r="AN108" s="89"/>
       <c r="AO108" s="89"/>
     </row>
-    <row r="109" spans="35:41" x14ac:dyDescent="0.25">
+    <row r="109" spans="35:41" x14ac:dyDescent="0.35">
       <c r="AI109" s="80"/>
       <c r="AJ109" s="89"/>
       <c r="AK109" s="89"/>
@@ -17897,7 +17897,7 @@
       <c r="AN109" s="89"/>
       <c r="AO109" s="89"/>
     </row>
-    <row r="110" spans="35:41" x14ac:dyDescent="0.25">
+    <row r="110" spans="35:41" x14ac:dyDescent="0.35">
       <c r="AI110" s="80"/>
       <c r="AJ110" s="89"/>
       <c r="AK110" s="89"/>
@@ -17906,7 +17906,7 @@
       <c r="AN110" s="89"/>
       <c r="AO110" s="89"/>
     </row>
-    <row r="111" spans="35:41" x14ac:dyDescent="0.25">
+    <row r="111" spans="35:41" x14ac:dyDescent="0.35">
       <c r="AI111" s="80"/>
       <c r="AJ111" s="89"/>
       <c r="AK111" s="89"/>
@@ -17915,7 +17915,7 @@
       <c r="AN111" s="89"/>
       <c r="AO111" s="89"/>
     </row>
-    <row r="112" spans="35:41" x14ac:dyDescent="0.25">
+    <row r="112" spans="35:41" x14ac:dyDescent="0.35">
       <c r="AI112" s="80"/>
       <c r="AJ112" s="89"/>
       <c r="AK112" s="89"/>
@@ -17924,7 +17924,7 @@
       <c r="AN112" s="89"/>
       <c r="AO112" s="89"/>
     </row>
-    <row r="113" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="113" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI113" s="80"/>
       <c r="AJ113" s="89"/>
       <c r="AK113" s="89"/>
@@ -17933,7 +17933,7 @@
       <c r="AN113" s="89"/>
       <c r="AO113" s="89"/>
     </row>
-    <row r="114" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="114" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI114" s="80"/>
       <c r="AJ114" s="89"/>
       <c r="AK114" s="89"/>
@@ -17942,7 +17942,7 @@
       <c r="AN114" s="89"/>
       <c r="AO114" s="89"/>
     </row>
-    <row r="115" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="115" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI115" s="80"/>
       <c r="AJ115" s="89"/>
       <c r="AK115" s="89"/>
@@ -17951,7 +17951,7 @@
       <c r="AN115" s="89"/>
       <c r="AO115" s="89"/>
     </row>
-    <row r="116" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="116" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI116" s="80"/>
       <c r="AJ116" s="89"/>
       <c r="AK116" s="89"/>
@@ -17960,7 +17960,7 @@
       <c r="AN116" s="89"/>
       <c r="AO116" s="89"/>
     </row>
-    <row r="117" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="117" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI117" s="80"/>
       <c r="AJ117" s="89"/>
       <c r="AK117" s="89"/>
@@ -17969,7 +17969,7 @@
       <c r="AN117" s="89"/>
       <c r="AO117" s="89"/>
     </row>
-    <row r="118" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="118" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI118" s="80"/>
       <c r="AJ118" s="89"/>
       <c r="AK118" s="89"/>
@@ -17978,7 +17978,7 @@
       <c r="AN118" s="89"/>
       <c r="AO118" s="89"/>
     </row>
-    <row r="119" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="119" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI119" s="80"/>
       <c r="AJ119" s="89"/>
       <c r="AK119" s="89"/>
@@ -17987,7 +17987,7 @@
       <c r="AN119" s="89"/>
       <c r="AO119" s="89"/>
     </row>
-    <row r="120" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="120" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI120" s="80"/>
       <c r="AJ120" s="89"/>
       <c r="AK120" s="89"/>
@@ -17996,7 +17996,7 @@
       <c r="AN120" s="89"/>
       <c r="AO120" s="89"/>
     </row>
-    <row r="121" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="121" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI121" s="80"/>
       <c r="AJ121" s="89"/>
       <c r="AK121" s="89"/>
@@ -18005,7 +18005,7 @@
       <c r="AN121" s="89"/>
       <c r="AO121" s="89"/>
     </row>
-    <row r="122" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="122" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI122" s="80"/>
       <c r="AJ122" s="89"/>
       <c r="AK122" s="89"/>
@@ -18014,7 +18014,7 @@
       <c r="AN122" s="89"/>
       <c r="AO122" s="89"/>
     </row>
-    <row r="123" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="123" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI123" s="80"/>
       <c r="AJ123" s="89"/>
       <c r="AK123" s="89"/>
@@ -18024,7 +18024,7 @@
       <c r="AO123" s="89"/>
       <c r="AP123" s="88"/>
     </row>
-    <row r="124" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="124" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI124" s="80"/>
       <c r="AJ124" s="89"/>
       <c r="AK124" s="89"/>
@@ -18033,7 +18033,7 @@
       <c r="AN124" s="89"/>
       <c r="AO124" s="89"/>
     </row>
-    <row r="125" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="125" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI125" s="80"/>
       <c r="AJ125" s="89"/>
       <c r="AK125" s="89"/>
@@ -18042,7 +18042,7 @@
       <c r="AN125" s="89"/>
       <c r="AO125" s="89"/>
     </row>
-    <row r="126" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="126" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI126" s="80"/>
       <c r="AJ126" s="89"/>
       <c r="AK126" s="89"/>
@@ -18051,7 +18051,7 @@
       <c r="AN126" s="89"/>
       <c r="AO126" s="89"/>
     </row>
-    <row r="127" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="127" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI127" s="80"/>
       <c r="AJ127" s="89"/>
       <c r="AK127" s="89"/>
@@ -18060,7 +18060,7 @@
       <c r="AN127" s="89"/>
       <c r="AO127" s="89"/>
     </row>
-    <row r="128" spans="35:42" x14ac:dyDescent="0.25">
+    <row r="128" spans="35:42" x14ac:dyDescent="0.35">
       <c r="AI128" s="80"/>
       <c r="AJ128" s="89"/>
       <c r="AK128" s="89"/>
@@ -18074,16 +18074,11 @@
     <protectedRange sqref="D30" name="Range1"/>
   </protectedRanges>
   <mergeCells count="31">
-    <mergeCell ref="O67:R67"/>
-    <mergeCell ref="D80:E80"/>
-    <mergeCell ref="D82:E82"/>
-    <mergeCell ref="D83:H83"/>
-    <mergeCell ref="D89:H89"/>
-    <mergeCell ref="D42:H42"/>
-    <mergeCell ref="D43:H43"/>
-    <mergeCell ref="D45:H45"/>
-    <mergeCell ref="E55:H55"/>
-    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="G16:H16"/>
+    <mergeCell ref="G17:H17"/>
+    <mergeCell ref="G18:H18"/>
     <mergeCell ref="G14:H14"/>
     <mergeCell ref="C23:I23"/>
     <mergeCell ref="B24:B25"/>
@@ -18100,11 +18095,16 @@
     <mergeCell ref="D39:H39"/>
     <mergeCell ref="D36:H36"/>
     <mergeCell ref="D40:H40"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
-    <mergeCell ref="G16:H16"/>
-    <mergeCell ref="G17:H17"/>
-    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="D43:H43"/>
+    <mergeCell ref="D45:H45"/>
+    <mergeCell ref="E55:H55"/>
+    <mergeCell ref="B33:I33"/>
+    <mergeCell ref="O67:R67"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="D82:E82"/>
+    <mergeCell ref="D83:H83"/>
+    <mergeCell ref="D89:H89"/>
   </mergeCells>
   <conditionalFormatting sqref="C28:C29">
     <cfRule type="cellIs" dxfId="21" priority="2" operator="greaterThan">
@@ -18244,7 +18244,7 @@
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>638175</xdr:colOff>
+                    <xdr:colOff>635000</xdr:colOff>
                     <xdr:row>33</xdr:row>
                     <xdr:rowOff>266700</xdr:rowOff>
                   </to>
@@ -18260,7 +18260,7 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>733425</xdr:colOff>
+                    <xdr:colOff>736600</xdr:colOff>
                     <xdr:row>33</xdr:row>
                     <xdr:rowOff>57150</xdr:rowOff>
                   </from>
@@ -18284,13 +18284,13 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>0</xdr:colOff>
                     <xdr:row>34</xdr:row>
-                    <xdr:rowOff>66675</xdr:rowOff>
+                    <xdr:rowOff>69850</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>638175</xdr:colOff>
+                    <xdr:colOff>641350</xdr:colOff>
                     <xdr:row>34</xdr:row>
-                    <xdr:rowOff>276225</xdr:rowOff>
+                    <xdr:rowOff>279400</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18304,15 +18304,15 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>733425</xdr:colOff>
+                    <xdr:colOff>736600</xdr:colOff>
                     <xdr:row>34</xdr:row>
-                    <xdr:rowOff>66675</xdr:rowOff>
+                    <xdr:rowOff>69850</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>1371600</xdr:colOff>
                     <xdr:row>34</xdr:row>
-                    <xdr:rowOff>276225</xdr:rowOff>
+                    <xdr:rowOff>279400</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18326,7 +18326,7 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>7</xdr:col>
-                    <xdr:colOff>123825</xdr:colOff>
+                    <xdr:colOff>127000</xdr:colOff>
                     <xdr:row>79</xdr:row>
                     <xdr:rowOff>38100</xdr:rowOff>
                   </from>
@@ -18334,7 +18334,7 @@
                     <xdr:col>7</xdr:col>
                     <xdr:colOff>990600</xdr:colOff>
                     <xdr:row>79</xdr:row>
-                    <xdr:rowOff>257175</xdr:rowOff>
+                    <xdr:rowOff>260350</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18356,7 +18356,7 @@
                     <xdr:col>8</xdr:col>
                     <xdr:colOff>552450</xdr:colOff>
                     <xdr:row>79</xdr:row>
-                    <xdr:rowOff>257175</xdr:rowOff>
+                    <xdr:rowOff>260350</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18370,9 +18370,9 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>7</xdr:col>
-                    <xdr:colOff>123825</xdr:colOff>
+                    <xdr:colOff>127000</xdr:colOff>
                     <xdr:row>80</xdr:row>
-                    <xdr:rowOff>66675</xdr:rowOff>
+                    <xdr:rowOff>69850</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>7</xdr:col>
@@ -18394,7 +18394,7 @@
                     <xdr:col>7</xdr:col>
                     <xdr:colOff>1066800</xdr:colOff>
                     <xdr:row>80</xdr:row>
-                    <xdr:rowOff>66675</xdr:rowOff>
+                    <xdr:rowOff>69850</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>8</xdr:col>
@@ -18414,13 +18414,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>4</xdr:col>
-                    <xdr:colOff>123825</xdr:colOff>
+                    <xdr:colOff>127000</xdr:colOff>
                     <xdr:row>80</xdr:row>
-                    <xdr:rowOff>66675</xdr:rowOff>
+                    <xdr:rowOff>69850</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>200025</xdr:colOff>
+                    <xdr:colOff>203200</xdr:colOff>
                     <xdr:row>81</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -18436,13 +18436,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>390525</xdr:colOff>
+                    <xdr:colOff>393700</xdr:colOff>
                     <xdr:row>80</xdr:row>
-                    <xdr:rowOff>66675</xdr:rowOff>
+                    <xdr:rowOff>69850</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>847725</xdr:colOff>
+                    <xdr:colOff>850900</xdr:colOff>
                     <xdr:row>81</xdr:row>
                     <xdr:rowOff>0</xdr:rowOff>
                   </to>
@@ -18458,9 +18458,9 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>942975</xdr:colOff>
+                    <xdr:colOff>946150</xdr:colOff>
                     <xdr:row>80</xdr:row>
-                    <xdr:rowOff>66675</xdr:rowOff>
+                    <xdr:rowOff>69850</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>6</xdr:col>
@@ -18486,9 +18486,9 @@
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>638175</xdr:colOff>
+                    <xdr:colOff>641350</xdr:colOff>
                     <xdr:row>40</xdr:row>
-                    <xdr:rowOff>276225</xdr:rowOff>
+                    <xdr:rowOff>279400</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18510,7 +18510,7 @@
                     <xdr:col>3</xdr:col>
                     <xdr:colOff>1181100</xdr:colOff>
                     <xdr:row>40</xdr:row>
-                    <xdr:rowOff>276225</xdr:rowOff>
+                    <xdr:rowOff>279400</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18530,9 +18530,9 @@
                   </from>
                   <to>
                     <xdr:col>5</xdr:col>
-                    <xdr:colOff>104775</xdr:colOff>
+                    <xdr:colOff>107950</xdr:colOff>
                     <xdr:row>40</xdr:row>
-                    <xdr:rowOff>276225</xdr:rowOff>
+                    <xdr:rowOff>279400</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18554,7 +18554,7 @@
                     <xdr:col>6</xdr:col>
                     <xdr:colOff>381000</xdr:colOff>
                     <xdr:row>40</xdr:row>
-                    <xdr:rowOff>276225</xdr:rowOff>
+                    <xdr:rowOff>279400</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18570,7 +18570,7 @@
                     <xdr:col>5</xdr:col>
                     <xdr:colOff>304800</xdr:colOff>
                     <xdr:row>61</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>31750</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>5</xdr:col>
@@ -18592,7 +18592,7 @@
                     <xdr:col>6</xdr:col>
                     <xdr:colOff>76200</xdr:colOff>
                     <xdr:row>61</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>31750</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>6</xdr:col>
@@ -18612,13 +18612,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>7</xdr:col>
-                    <xdr:colOff>314325</xdr:colOff>
+                    <xdr:colOff>317500</xdr:colOff>
                     <xdr:row>61</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>31750</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>7</xdr:col>
-                    <xdr:colOff>600075</xdr:colOff>
+                    <xdr:colOff>603250</xdr:colOff>
                     <xdr:row>61</xdr:row>
                     <xdr:rowOff>247650</xdr:rowOff>
                   </to>
@@ -18634,9 +18634,9 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>7</xdr:col>
-                    <xdr:colOff>1419225</xdr:colOff>
+                    <xdr:colOff>1422400</xdr:colOff>
                     <xdr:row>61</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>31750</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>8</xdr:col>
@@ -18658,7 +18658,7 @@
                     <xdr:col>9</xdr:col>
                     <xdr:colOff>0</xdr:colOff>
                     <xdr:row>61</xdr:row>
-                    <xdr:rowOff>28575</xdr:rowOff>
+                    <xdr:rowOff>31750</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>9</xdr:col>
@@ -18684,9 +18684,9 @@
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>638175</xdr:colOff>
+                    <xdr:colOff>641350</xdr:colOff>
                     <xdr:row>39</xdr:row>
-                    <xdr:rowOff>257175</xdr:rowOff>
+                    <xdr:rowOff>260350</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18706,9 +18706,9 @@
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>1362075</xdr:colOff>
+                    <xdr:colOff>1365250</xdr:colOff>
                     <xdr:row>39</xdr:row>
-                    <xdr:rowOff>257175</xdr:rowOff>
+                    <xdr:rowOff>260350</xdr:rowOff>
                   </to>
                 </anchor>
               </controlPr>
@@ -18722,13 +18722,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>257175</xdr:colOff>
+                    <xdr:colOff>260350</xdr:colOff>
                     <xdr:row>14</xdr:row>
                     <xdr:rowOff>38100</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>933450</xdr:colOff>
+                    <xdr:colOff>965200</xdr:colOff>
                     <xdr:row>14</xdr:row>
                     <xdr:rowOff>247650</xdr:rowOff>
                   </to>
@@ -18744,13 +18744,13 @@
                 <anchor moveWithCells="1">
                   <from>
                     <xdr:col>2</xdr:col>
-                    <xdr:colOff>1047750</xdr:colOff>
+                    <xdr:colOff>1073150</xdr:colOff>
                     <xdr:row>14</xdr:row>
                     <xdr:rowOff>38100</xdr:rowOff>
                   </from>
                   <to>
                     <xdr:col>3</xdr:col>
-                    <xdr:colOff>485775</xdr:colOff>
+                    <xdr:colOff>488950</xdr:colOff>
                     <xdr:row>14</xdr:row>
                     <xdr:rowOff>247650</xdr:rowOff>
                   </to>
@@ -18768,12 +18768,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="94" t="s">
         <v>226</v>
       </c>
@@ -18784,7 +18784,7 @@
       <c r="D1" s="94"/>
       <c r="E1" s="94"/>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="94" t="s">
         <v>228</v>
       </c>
@@ -18804,50 +18804,49 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.5703125" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9.140625" style="2"/>
-    <col min="3" max="3" width="13.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="21.7109375" style="2" customWidth="1"/>
-    <col min="5" max="6" width="9.140625" style="2"/>
-    <col min="7" max="8" width="11" style="91" customWidth="1"/>
-    <col min="9" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="18.54296875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="13.7265625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="21.7265625" style="2" customWidth="1"/>
+    <col min="4" max="5" width="9.1796875" style="2"/>
+    <col min="6" max="7" width="11" style="91" customWidth="1"/>
+    <col min="8" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="94" t="s">
         <v>230</v>
       </c>
+      <c r="F1" s="91" t="s">
+        <v>237</v>
+      </c>
       <c r="G1" s="91" t="s">
-        <v>237</v>
-      </c>
-      <c r="H1" s="91" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="94"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="156" t="s">
         <v>231</v>
       </c>
       <c r="B3" s="156" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="C3" s="156" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D3" s="156" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="E3" s="156" t="s">
         <v>235</v>
       </c>
-      <c r="F3" s="156" t="s">
-        <v>236</v>
+      <c r="I3" s="156" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
@@ -18858,50 +18857,51 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B3:AH49"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B3:S25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="3" spans="2:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:19" x14ac:dyDescent="0.35">
       <c r="B3" s="156" t="s">
         <v>241</v>
       </c>
-      <c r="AA3" s="156" t="s">
+      <c r="S3" s="156" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="49" spans="34:34" x14ac:dyDescent="0.25">
-      <c r="AH49" s="156" t="s">
+    <row r="25" spans="19:19" x14ac:dyDescent="0.35">
+      <c r="S25" s="156" t="s">
         <v>243</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="B1:V45"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="6.7109375" style="2" customWidth="1"/>
-    <col min="2" max="2" width="5.28515625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="29.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="9.140625" style="2"/>
-    <col min="5" max="11" width="10.85546875" style="2" customWidth="1"/>
-    <col min="12" max="13" width="4.140625" style="2" customWidth="1"/>
-    <col min="14" max="14" width="29.7109375" style="2" customWidth="1"/>
-    <col min="15" max="15" width="9.140625" style="2"/>
-    <col min="16" max="22" width="9.28515625" style="2" customWidth="1"/>
-    <col min="23" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="6.7265625" style="2" customWidth="1"/>
+    <col min="2" max="2" width="5.26953125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="29.7265625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="9.1796875" style="2"/>
+    <col min="5" max="11" width="10.81640625" style="2" customWidth="1"/>
+    <col min="12" max="13" width="4.1796875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="29.7265625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="9.1796875" style="2"/>
+    <col min="16" max="22" width="9.26953125" style="2" customWidth="1"/>
+    <col min="23" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:22" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:22" ht="22.5" customHeight="1" x14ac:dyDescent="0.4">
       <c r="B1" s="1" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>297</v>
@@ -18910,7 +18910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="K2" s="5" t="s">
         <v>276</v>
       </c>
@@ -18918,7 +18918,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="3" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="90"/>
       <c r="C3" s="90"/>
       <c r="D3" s="90"/>
@@ -18934,7 +18934,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="90"/>
       <c r="C4" s="90"/>
       <c r="D4" s="90"/>
@@ -18950,7 +18950,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="90"/>
       <c r="C5" s="90"/>
       <c r="D5" s="90"/>
@@ -18966,7 +18966,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="90"/>
       <c r="C6" s="90"/>
       <c r="D6" s="90"/>
@@ -18982,7 +18982,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="90"/>
       <c r="C7" s="90"/>
       <c r="D7" s="90"/>
@@ -18998,7 +18998,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="90"/>
       <c r="C8" s="90"/>
       <c r="D8" s="90"/>
@@ -19008,7 +19008,7 @@
       <c r="H8" s="90"/>
       <c r="I8" s="90"/>
     </row>
-    <row r="9" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:22" ht="17.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="90"/>
       <c r="C9" s="90"/>
       <c r="D9" s="90"/>
@@ -19021,11 +19021,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="2:22" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:22" ht="7.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="O10" s="8"/>
     </row>
-    <row r="11" spans="2:22" ht="22.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="2:22" ht="18" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:22" ht="22.5" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="12" spans="2:22" ht="18" x14ac:dyDescent="0.4">
       <c r="C12" s="9" t="s">
         <v>9</v>
       </c>
@@ -19046,7 +19046,7 @@
       <c r="U12" s="15"/>
       <c r="V12" s="15"/>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B13" s="15"/>
       <c r="C13" s="16"/>
       <c r="D13" s="238"/>
@@ -19068,7 +19068,7 @@
       <c r="U13" s="18"/>
       <c r="V13" s="18"/>
     </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B14" s="18"/>
       <c r="C14" s="20"/>
       <c r="D14" s="21"/>
@@ -19102,29 +19102,29 @@
       <c r="U14" s="23"/>
       <c r="V14" s="23"/>
     </row>
-    <row r="15" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B15" s="24"/>
       <c r="C15" s="318" t="s">
         <v>10</v>
       </c>
       <c r="D15" s="319"/>
       <c r="E15" s="25">
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="F15" s="25">
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="G15" s="25">
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="H15" s="25">
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="I15" s="25">
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="J15" s="25">
-        <v>15</v>
+        <v>18.5</v>
       </c>
       <c r="L15" s="24"/>
       <c r="M15" s="24"/>
@@ -19138,7 +19138,7 @@
       <c r="U15" s="26"/>
       <c r="V15" s="26"/>
     </row>
-    <row r="16" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B16" s="24"/>
       <c r="C16" s="27"/>
       <c r="D16" s="24"/>
@@ -19160,7 +19160,7 @@
       <c r="U16" s="26"/>
       <c r="V16" s="26"/>
     </row>
-    <row r="17" spans="2:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:22" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B17" s="15"/>
       <c r="C17" s="28" t="s">
         <v>11</v>
@@ -19186,7 +19186,7 @@
       <c r="U17" s="30"/>
       <c r="V17" s="30"/>
     </row>
-    <row r="18" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B18" s="15"/>
       <c r="C18" s="32"/>
       <c r="D18" s="33"/>
@@ -19208,7 +19208,7 @@
       <c r="U18" s="30"/>
       <c r="V18" s="30"/>
     </row>
-    <row r="19" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B19" s="15"/>
       <c r="C19" s="37" t="s">
         <v>12</v>
@@ -19216,27 +19216,27 @@
       <c r="D19" s="38"/>
       <c r="E19" s="39">
         <f t="shared" ref="E19:J19" si="0">$D$17*E15</f>
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="F19" s="39">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="G19" s="39">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="H19" s="39">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="I19" s="39">
         <f t="shared" si="0"/>
-        <v>17</v>
+        <v>18.5</v>
       </c>
       <c r="J19" s="39">
         <f t="shared" si="0"/>
-        <v>15</v>
+        <v>18.5</v>
       </c>
       <c r="L19" s="15"/>
       <c r="M19" s="15"/>
@@ -19250,7 +19250,7 @@
       <c r="U19" s="26"/>
       <c r="V19" s="26"/>
     </row>
-    <row r="20" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B20" s="15"/>
       <c r="C20" s="40" t="s">
         <v>13</v>
@@ -19286,7 +19286,7 @@
       <c r="U20" s="26"/>
       <c r="V20" s="26"/>
     </row>
-    <row r="21" spans="2:22" s="47" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:22" s="47" customFormat="1" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B21" s="43"/>
       <c r="C21" s="44" t="s">
         <v>14</v>
@@ -19294,27 +19294,27 @@
       <c r="D21" s="45"/>
       <c r="E21" s="46">
         <f>E20+E19</f>
-        <v>44</v>
+        <v>45.5</v>
       </c>
       <c r="F21" s="46">
         <f t="shared" ref="F21:J21" si="1">F20+F19</f>
-        <v>44</v>
+        <v>45.5</v>
       </c>
       <c r="G21" s="46">
         <f t="shared" si="1"/>
-        <v>44</v>
+        <v>45.5</v>
       </c>
       <c r="H21" s="46">
         <f t="shared" si="1"/>
-        <v>44</v>
+        <v>45.5</v>
       </c>
       <c r="I21" s="46">
         <f t="shared" si="1"/>
-        <v>44</v>
+        <v>45.5</v>
       </c>
       <c r="J21" s="46">
         <f t="shared" si="1"/>
-        <v>42</v>
+        <v>45.5</v>
       </c>
       <c r="L21" s="43"/>
       <c r="M21" s="43"/>
@@ -19328,7 +19328,7 @@
       <c r="U21" s="50"/>
       <c r="V21" s="50"/>
     </row>
-    <row r="22" spans="2:22" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:22" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B22" s="27"/>
       <c r="C22" s="27"/>
       <c r="D22" s="24"/>
@@ -19350,7 +19350,7 @@
       <c r="U22" s="51"/>
       <c r="V22" s="51"/>
     </row>
-    <row r="23" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C23" s="53"/>
       <c r="D23" s="53"/>
       <c r="E23" s="52"/>
@@ -19369,7 +19369,7 @@
       <c r="U23" s="52"/>
       <c r="V23" s="52"/>
     </row>
-    <row r="24" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C24" s="53"/>
       <c r="D24" s="53"/>
       <c r="E24" s="52"/>
@@ -19389,7 +19389,7 @@
       <c r="U24" s="52"/>
       <c r="V24" s="52"/>
     </row>
-    <row r="25" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:22" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="C25" s="53"/>
       <c r="D25" s="53"/>
       <c r="E25" s="52"/>
@@ -19409,7 +19409,7 @@
       <c r="U25" s="52"/>
       <c r="V25" s="52"/>
     </row>
-    <row r="26" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B26" s="27"/>
       <c r="C26" s="27"/>
       <c r="D26" s="24"/>
@@ -19421,7 +19421,7 @@
       <c r="J26" s="51"/>
       <c r="K26" s="51"/>
     </row>
-    <row r="27" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B27" s="27"/>
       <c r="C27" s="27"/>
       <c r="D27" s="27"/>
@@ -19433,7 +19433,7 @@
       <c r="J27" s="54"/>
       <c r="K27" s="54"/>
     </row>
-    <row r="28" spans="2:22" ht="18" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:22" ht="18" x14ac:dyDescent="0.4">
       <c r="C28" s="9" t="s">
         <v>15</v>
       </c>
@@ -19454,7 +19454,7 @@
       <c r="U28" s="54"/>
       <c r="V28" s="54"/>
     </row>
-    <row r="29" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B29" s="15"/>
       <c r="C29" s="252"/>
       <c r="D29" s="253"/>
@@ -19474,7 +19474,7 @@
       <c r="U29" s="60"/>
       <c r="V29" s="60"/>
     </row>
-    <row r="30" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B30" s="27"/>
       <c r="C30" s="256"/>
       <c r="D30" s="257"/>
@@ -19506,7 +19506,7 @@
       <c r="U30" s="23"/>
       <c r="V30" s="23"/>
     </row>
-    <row r="31" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B31" s="24"/>
       <c r="C31" s="318" t="str">
         <f>C15</f>
@@ -19514,22 +19514,22 @@
       </c>
       <c r="D31" s="319"/>
       <c r="E31" s="61">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="F31" s="61">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="G31" s="61">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="H31" s="61">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="I31" s="61">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J31" s="61">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="N31" s="320"/>
       <c r="O31" s="320"/>
@@ -19541,7 +19541,7 @@
       <c r="U31" s="26"/>
       <c r="V31" s="26"/>
     </row>
-    <row r="32" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B32" s="24"/>
       <c r="C32" s="15"/>
       <c r="D32" s="15"/>
@@ -19561,10 +19561,10 @@
       <c r="U32" s="26"/>
       <c r="V32" s="26"/>
     </row>
-    <row r="33" spans="2:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:22" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B33" s="24"/>
       <c r="C33" s="258" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D33" s="259">
         <v>1</v>
@@ -19574,7 +19574,7 @@
         <v>5</v>
       </c>
       <c r="F33" s="323" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G33" s="260"/>
       <c r="H33" s="260"/>
@@ -19590,7 +19590,7 @@
       <c r="U33" s="30"/>
       <c r="V33" s="30"/>
     </row>
-    <row r="34" spans="2:22" ht="30" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:22" ht="29" x14ac:dyDescent="0.35">
       <c r="B34" s="24"/>
       <c r="C34" s="261" t="s">
         <v>20</v>
@@ -19614,7 +19614,7 @@
       <c r="U34" s="30"/>
       <c r="V34" s="30"/>
     </row>
-    <row r="35" spans="2:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:22" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B35" s="24"/>
       <c r="C35" s="236" t="s">
         <v>21</v>
@@ -19627,7 +19627,7 @@
         <v>0</v>
       </c>
       <c r="F35" s="264" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G35" s="30"/>
       <c r="H35" s="30"/>
@@ -19643,7 +19643,7 @@
       <c r="U35" s="26"/>
       <c r="V35" s="26"/>
     </row>
-    <row r="36" spans="2:22" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:22" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B36" s="24"/>
       <c r="C36" s="236" t="s">
         <v>67</v>
@@ -19656,7 +19656,7 @@
         <v>0</v>
       </c>
       <c r="F36" s="264" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G36" s="30"/>
       <c r="H36" s="30"/>
@@ -19672,10 +19672,10 @@
       <c r="U36" s="26"/>
       <c r="V36" s="26"/>
     </row>
-    <row r="37" spans="2:22" s="47" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:22" s="47" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
       <c r="B37" s="62"/>
       <c r="C37" s="265" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D37" s="266">
         <f>D33*D34+D35+D36</f>
@@ -19686,7 +19686,7 @@
         <v>5</v>
       </c>
       <c r="F37" s="268" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="G37" s="30"/>
       <c r="H37" s="30"/>
@@ -19702,7 +19702,7 @@
       <c r="U37" s="50"/>
       <c r="V37" s="50"/>
     </row>
-    <row r="38" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B38" s="24"/>
       <c r="C38" s="32"/>
       <c r="D38" s="33"/>
@@ -19723,7 +19723,7 @@
       <c r="U38" s="63"/>
       <c r="V38" s="63"/>
     </row>
-    <row r="39" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B39" s="24"/>
       <c r="C39" s="37" t="s">
         <v>12</v>
@@ -19731,31 +19731,31 @@
       <c r="D39" s="38"/>
       <c r="E39" s="39">
         <f>$E$37*E31</f>
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="F39" s="39">
         <f t="shared" ref="F39:J39" si="2">$E$37*F31</f>
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="G39" s="39">
         <f t="shared" si="2"/>
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="H39" s="39">
         <f t="shared" si="2"/>
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="I39" s="39">
         <f t="shared" si="2"/>
-        <v>170</v>
+        <v>185</v>
       </c>
       <c r="J39" s="39">
         <f t="shared" si="2"/>
-        <v>150</v>
+        <v>185</v>
       </c>
       <c r="K39" s="63"/>
     </row>
-    <row r="40" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B40" s="24"/>
       <c r="C40" s="40" t="s">
         <v>13</v>
@@ -19781,7 +19781,7 @@
       </c>
       <c r="K40" s="63"/>
     </row>
-    <row r="41" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="2:22" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B41" s="24"/>
       <c r="C41" s="44" t="str">
         <f>C21</f>
@@ -19790,31 +19790,31 @@
       <c r="D41" s="45"/>
       <c r="E41" s="46">
         <f t="shared" ref="E41" si="3">E40+E39</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="F41" s="46">
         <f>F40+F39</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="G41" s="46">
         <f>G40+G39</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="H41" s="46">
         <f>H40+H39</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="I41" s="46">
         <f>I40+I39</f>
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="J41" s="46">
         <f>J40+J39</f>
-        <v>177</v>
+        <v>212</v>
       </c>
       <c r="K41" s="63"/>
     </row>
-    <row r="42" spans="2:22" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:22" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="B42" s="24"/>
       <c r="C42" s="27"/>
       <c r="D42" s="24"/>
@@ -19826,7 +19826,7 @@
       <c r="J42" s="63"/>
       <c r="K42" s="63"/>
     </row>
-    <row r="43" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B43" s="24"/>
       <c r="C43" s="27"/>
       <c r="D43" s="24"/>
@@ -19838,10 +19838,10 @@
       <c r="J43" s="63"/>
       <c r="K43" s="63"/>
     </row>
-    <row r="44" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B44" s="24"/>
     </row>
-    <row r="45" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:22" x14ac:dyDescent="0.35">
       <c r="B45" s="24"/>
     </row>
   </sheetData>
@@ -19868,18 +19868,18 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:L54"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.85546875" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="29.81640625" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" s="65" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="65" customFormat="1" ht="35.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="152" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="65" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" s="65" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="153" t="s">
         <v>87</v>
       </c>
@@ -19887,39 +19887,39 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:12" s="65" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" s="65" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="153"/>
       <c r="B3" s="68" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="4" spans="1:12" s="65" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" s="65" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B4" s="2" t="s">
         <v>252</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="86" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" s="86" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B6" s="154" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="314" t="s">
+    <row r="7" spans="1:12" s="154" customFormat="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B8" s="299" t="s">
         <v>91</v>
       </c>
-      <c r="C8" s="314"/>
-      <c r="D8" s="314"/>
-      <c r="E8" s="314"/>
-      <c r="F8" s="314"/>
-      <c r="G8" s="314"/>
-      <c r="H8" s="314"/>
-      <c r="I8" s="314"/>
-      <c r="J8" s="314"/>
-      <c r="K8" s="314"/>
-      <c r="L8" s="314"/>
-    </row>
-    <row r="9" spans="1:12" ht="100.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="299"/>
+      <c r="D8" s="299"/>
+      <c r="E8" s="299"/>
+      <c r="F8" s="299"/>
+      <c r="G8" s="299"/>
+      <c r="H8" s="299"/>
+      <c r="I8" s="299"/>
+      <c r="J8" s="299"/>
+      <c r="K8" s="299"/>
+      <c r="L8" s="299"/>
+    </row>
+    <row r="9" spans="1:12" ht="100.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="325" t="s">
         <v>253</v>
       </c>
@@ -19934,7 +19934,7 @@
       <c r="K9" s="325"/>
       <c r="L9" s="325"/>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B10" s="326" t="s">
         <v>92</v>
       </c>
@@ -19947,7 +19947,7 @@
       <c r="I10" s="326"/>
       <c r="J10" s="326"/>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B11" s="155"/>
       <c r="C11" s="155"/>
       <c r="D11" s="155"/>
@@ -19958,7 +19958,7 @@
       <c r="I11" s="155"/>
       <c r="J11" s="155"/>
     </row>
-    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="156" t="s">
         <v>93</v>
       </c>
@@ -19966,7 +19966,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="327" t="s">
         <v>95</v>
       </c>
@@ -19981,7 +19981,7 @@
       <c r="K14" s="327"/>
       <c r="L14" s="327"/>
     </row>
-    <row r="15" spans="1:12" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:12" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="325" t="s">
         <v>96</v>
       </c>
@@ -19996,7 +19996,7 @@
       <c r="K15" s="325"/>
       <c r="L15" s="325"/>
     </row>
-    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="325" t="s">
         <v>97</v>
       </c>
@@ -20011,17 +20011,17 @@
       <c r="K16" s="325"/>
       <c r="L16" s="325"/>
     </row>
-    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="157" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B18" s="157" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="19" spans="1:12" s="65" customFormat="1" ht="80.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:12" s="65" customFormat="1" ht="80.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="325" t="s">
         <v>100</v>
       </c>
@@ -20036,7 +20036,7 @@
       <c r="K19" s="325"/>
       <c r="L19" s="325"/>
     </row>
-    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>101</v>
       </c>
@@ -20053,10 +20053,10 @@
       <c r="K20" s="158"/>
       <c r="L20" s="158"/>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
       <c r="B21" s="157"/>
     </row>
-    <row r="23" spans="1:12" s="108" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:12" s="108" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="A23" s="108" t="s">
         <v>103</v>
       </c>
@@ -20064,30 +20064,30 @@
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:12" s="108" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:12" s="108" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B24" s="2" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="1:12" s="108" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:12" s="108" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B25" s="2" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="26" spans="1:12" s="108" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:12" s="108" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B26" s="2" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="108" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:12" s="108" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B27" s="2" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="28" spans="1:12" s="108" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:12" s="108" customFormat="1" ht="18.5" x14ac:dyDescent="0.45">
       <c r="B28" s="2"/>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>109</v>
       </c>
@@ -20098,7 +20098,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>112</v>
       </c>
@@ -20109,7 +20109,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>115</v>
       </c>
@@ -20117,7 +20117,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>117</v>
       </c>
@@ -20125,7 +20125,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" s="160" t="s">
         <v>119</v>
       </c>
@@ -20133,12 +20133,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D35" s="2" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>122</v>
       </c>
@@ -20146,77 +20146,77 @@
         <v>123</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D40" s="2" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D41" s="2" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D42" s="2" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D43" s="2" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D44" s="2" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D45" s="2" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D46" s="2" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D47" s="2" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D48" s="2" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="49" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D49" s="2" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="50" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D50" s="2" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="51" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D51" s="2" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="52" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D52" s="2" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="53" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D53" s="2" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D54" s="2" t="s">
         <v>138</v>
       </c>
@@ -20249,24 +20249,24 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H65"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="30.28515625" style="2" customWidth="1"/>
-    <col min="2" max="16384" width="9.140625" style="2"/>
+    <col min="1" max="1" width="30.26953125" style="2" customWidth="1"/>
+    <col min="2" max="16384" width="9.1796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="161" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="5" spans="1:8" ht="31.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
+    <row r="5" spans="1:8" ht="30" thickTop="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="162" t="s">
         <v>141</v>
       </c>
@@ -20290,8 +20290,8 @@
       </c>
       <c r="H5" s="328"/>
     </row>
-    <row r="6" spans="1:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="15" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A8" s="99" t="s">
         <v>148</v>
       </c>
@@ -20314,7 +20314,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="99" t="s">
         <v>151</v>
       </c>
@@ -20329,7 +20329,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>153</v>
       </c>
@@ -20352,7 +20352,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>155</v>
       </c>
@@ -20375,7 +20375,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>159</v>
       </c>
@@ -20398,7 +20398,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>161</v>
       </c>
@@ -20421,7 +20421,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="99" t="s">
         <v>163</v>
       </c>
@@ -20444,7 +20444,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="99" t="s">
         <v>164</v>
       </c>
@@ -20467,7 +20467,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="99" t="s">
         <v>166</v>
       </c>
@@ -20482,7 +20482,7 @@
       </c>
       <c r="G16" s="99"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>167</v>
       </c>
@@ -20505,7 +20505,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>170</v>
       </c>
@@ -20528,7 +20528,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>172</v>
       </c>
@@ -20551,7 +20551,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>173</v>
       </c>
@@ -20574,7 +20574,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
         <v>175</v>
       </c>
@@ -20597,7 +20597,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>176</v>
       </c>
@@ -20620,7 +20620,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>177</v>
       </c>
@@ -20643,7 +20643,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>178</v>
       </c>
@@ -20666,7 +20666,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>179</v>
       </c>
@@ -20689,7 +20689,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>181</v>
       </c>
@@ -20712,7 +20712,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>182</v>
       </c>
@@ -20732,7 +20732,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>184</v>
       </c>
@@ -20755,7 +20755,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>185</v>
       </c>
@@ -20778,7 +20778,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>186</v>
       </c>
@@ -20801,7 +20801,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>188</v>
       </c>
@@ -20824,7 +20824,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>190</v>
       </c>
@@ -20847,7 +20847,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>192</v>
       </c>
@@ -20870,7 +20870,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>193</v>
       </c>
@@ -20893,7 +20893,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>194</v>
       </c>
@@ -20916,7 +20916,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>196</v>
       </c>
@@ -20939,7 +20939,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>198</v>
       </c>
@@ -20962,7 +20962,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A38" s="99" t="s">
         <v>200</v>
       </c>
@@ -20985,7 +20985,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>201</v>
       </c>
@@ -21008,7 +21008,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>204</v>
       </c>
@@ -21031,7 +21031,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A41" s="99" t="s">
         <v>206</v>
       </c>
@@ -21054,7 +21054,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>207</v>
       </c>
@@ -21077,146 +21077,146 @@
         <v>208</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C43" s="168"/>
       <c r="D43" s="168"/>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
       <c r="C44" s="168"/>
       <c r="D44" s="168"/>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A45" s="99" t="s">
         <v>209</v>
       </c>
       <c r="C45" s="168"/>
       <c r="D45" s="168"/>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A46" s="99" t="s">
         <v>210</v>
       </c>
       <c r="C46" s="168"/>
       <c r="D46" s="168"/>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A47" s="99" t="s">
         <v>211</v>
       </c>
       <c r="C47" s="168"/>
       <c r="D47" s="168"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A48" s="99" t="s">
         <v>212</v>
       </c>
       <c r="C48" s="168"/>
       <c r="D48" s="168"/>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="99" t="s">
         <v>213</v>
       </c>
       <c r="C49" s="168"/>
       <c r="D49" s="168"/>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50" s="99" t="s">
         <v>214</v>
       </c>
       <c r="C50" s="168"/>
       <c r="D50" s="168"/>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51" s="99" t="s">
         <v>215</v>
       </c>
       <c r="C51" s="168"/>
       <c r="D51" s="168"/>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52" s="99" t="s">
         <v>216</v>
       </c>
       <c r="C52" s="168"/>
       <c r="D52" s="168"/>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53" s="99" t="s">
         <v>217</v>
       </c>
       <c r="C53" s="168"/>
       <c r="D53" s="168"/>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54" s="99" t="s">
         <v>218</v>
       </c>
       <c r="C54" s="168"/>
       <c r="D54" s="168"/>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55" s="169" t="s">
         <v>219</v>
       </c>
       <c r="C55" s="168"/>
       <c r="D55" s="168"/>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56" s="169" t="s">
         <v>220</v>
       </c>
       <c r="C56" s="168"/>
       <c r="D56" s="168"/>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57" s="99" t="s">
         <v>221</v>
       </c>
       <c r="C57" s="168"/>
       <c r="D57" s="168"/>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="169" t="s">
         <v>222</v>
       </c>
       <c r="C58" s="168"/>
       <c r="D58" s="168"/>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="169" t="s">
         <v>223</v>
       </c>
       <c r="C59" s="168"/>
       <c r="D59" s="168"/>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="169" t="s">
         <v>224</v>
       </c>
       <c r="C60" s="168"/>
       <c r="D60" s="168"/>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="99" t="s">
         <v>225</v>
       </c>
       <c r="C61" s="168"/>
       <c r="D61" s="168"/>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C62" s="168"/>
       <c r="D62" s="168"/>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C63" s="168"/>
       <c r="D63" s="168"/>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="C64" s="168"/>
       <c r="D64" s="168"/>
     </row>
-    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="3:4" x14ac:dyDescent="0.35">
       <c r="C65" s="168"/>
       <c r="D65" s="168"/>
     </row>

</xml_diff>